<commit_message>
Wiederherstellung reinzelliger Tabellen-Netzplan & PSP: Parallele Zweige (V10 || V11) vertikal gestaffelt, 100% native Excel-Zellen ohne Bildobjekt
</commit_message>
<xml_diff>
--- a/docs/01_Projektorganisation/Netzplan.xlsx
+++ b/docs/01_Projektorganisation/Netzplan.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,19 +29,8 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F497D"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00262626"/>
-      <sz val="10"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -53,6 +42,134 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5597"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00333333"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5597"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5597"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5597"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
@@ -94,14 +211,8 @@
       <color rgb="009C0006"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00404040"/>
-      <sz val="9.5"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -115,7 +226,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -125,7 +236,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DEEBF7"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -133,8 +244,28 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -156,54 +287,402 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E6B8B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E6B8B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E6B8B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E6B8B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E6B8B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E6B8B8"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C00000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E6B8B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E6B8B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E6B8B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E6B8B8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C00000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00C00000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E6B8B8"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C00000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E6B8B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E6B8B8"/>
+      </left>
+      <right style="medium">
+        <color rgb="00C00000"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C00000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E6B8B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00C00000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E6B8B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E6B8B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E6B8B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E6B8B8"/>
+      </left>
+      <right style="medium">
+        <color rgb="00C00000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E6B8B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E6B8B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00C00000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E6B8B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E6B8B8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C00000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E6B8B8"/>
+      </left>
+      <right style="medium">
+        <color rgb="00C00000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E6B8B8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C00000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="medium">
+        <color rgb="002F5597"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002F5597"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002F5597"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="medium">
+        <color rgb="002F5597"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="medium">
+        <color rgb="002F5597"/>
+      </right>
+      <top style="medium">
+        <color rgb="002F5597"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002F5597"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="medium">
+        <color rgb="002F5597"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="002F5597"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002F5597"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="medium">
+        <color rgb="002F5597"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002F5597"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -278,36 +757,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>7</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="10953750" cy="6505575"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -599,40 +1048,1114 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B6"/>
+  <dimension ref="B2:AM35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6.2" customWidth="1" min="1" max="1"/>
+    <col width="6.2" customWidth="1" min="2" max="2"/>
+    <col width="6.2" customWidth="1" min="3" max="3"/>
+    <col width="6.2" customWidth="1" min="4" max="4"/>
+    <col width="6.2" customWidth="1" min="5" max="5"/>
+    <col width="6.2" customWidth="1" min="6" max="6"/>
+    <col width="6.2" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="6.2" customWidth="1" min="10" max="10"/>
+    <col width="6.2" customWidth="1" min="11" max="11"/>
+    <col width="6.2" customWidth="1" min="12" max="12"/>
+    <col width="6.2" customWidth="1" min="13" max="13"/>
+    <col width="6.2" customWidth="1" min="14" max="14"/>
+    <col width="6.2" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="6.2" customWidth="1" min="18" max="18"/>
+    <col width="6.2" customWidth="1" min="19" max="19"/>
+    <col width="6.2" customWidth="1" min="20" max="20"/>
+    <col width="6.2" customWidth="1" min="21" max="21"/>
+    <col width="6.2" customWidth="1" min="22" max="22"/>
+    <col width="6.2" customWidth="1" min="23" max="23"/>
+    <col width="4" customWidth="1" min="24" max="24"/>
+    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="6.2" customWidth="1" min="26" max="26"/>
+    <col width="6.2" customWidth="1" min="27" max="27"/>
+    <col width="6.2" customWidth="1" min="28" max="28"/>
+    <col width="6.2" customWidth="1" min="29" max="29"/>
+    <col width="6.2" customWidth="1" min="30" max="30"/>
+    <col width="6.2" customWidth="1" min="31" max="31"/>
+    <col width="4" customWidth="1" min="32" max="32"/>
+    <col width="4" customWidth="1" min="33" max="33"/>
+    <col width="6.2" customWidth="1" min="34" max="34"/>
+    <col width="6.2" customWidth="1" min="35" max="35"/>
+    <col width="6.2" customWidth="1" min="36" max="36"/>
+    <col width="6.2" customWidth="1" min="37" max="37"/>
+    <col width="6.2" customWidth="1" min="38" max="38"/>
+    <col width="6.2" customWidth="1" min="39" max="39"/>
+    <col width="6.2" customWidth="1" min="40" max="40"/>
+    <col width="6.2" customWidth="1" min="41" max="41"/>
+    <col width="6.2" customWidth="1" min="42" max="42"/>
+    <col width="6.2" customWidth="1" min="43" max="43"/>
+    <col width="6.2" customWidth="1" min="44" max="44"/>
+  </cols>
   <sheetData>
-    <row r="2">
+    <row r="1" ht="12" customHeight="1"/>
+    <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Netzplan nach DIN 69900 (Knotenvorgangsmodell)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Netzplan nach DIN 69900 (Knotenvorgangsmodell CPM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Projekt: IT-Ausstattung VektorPlan GmbH | NextLevel IT Solutions GmbH | Gesamtlaufzeit: 46 Arbeitstage</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Projekt: IT-Ausstattung Planungs- und Konstruktionsbüro | Kunde: VektorPlan GmbH | Projektleiter: Jan Kluth | Gesamtdauer: 46 Arbeitstage</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="10" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Hinweis: Untenstehend ist der vollstaendige, hochaufloesende DIN 69900 Netzplan mit kritischem Pfad (rot) eingebettet.</t>
+          <t>Legende Vorgangsknoten (DIN 69900)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Erläuterung der Pfade &amp; Farben im Netzplan:</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Detaillierte Rechenschritte (Vorwaerts-/Rueckwaertsrechnung, Puffer) finden Sie im Tabellenblatt 'DIN 69900 Berechnungstabelle'.</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>FAZ (Früh. Start)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Dauer (Tage)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>FEZ (Früh. Ende)</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>■ KRITISCHER PFAD (Rot / Warmgelb): Gesamtpuffer GP = 0. Jede Verzögerung verschiebt unmittelbar das Projektende (Dauer: 46 Arbeitstage).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Vorgangs-Nr. &amp; Vorgangsbezeichnung (Kritisch = Roter Rahmen)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="n"/>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>■ PARALLELE VORGÄNGE &amp; PUFFER (Blau): V10 (Entsorgung Altdrucker) läuft parallel zu V11 (Montage). V10 hat 1 Tag Gesamtpuffer (GP = 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>SAZ (Spät. Start)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>GP (Gesamtpuffer)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>SEZ (Spät. Ende)</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="n"/>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>➔ Normalfolge (Ende-Anfang EA = 0): Der Nachfolger beginnt frühestens unmittelbar nach Beendigung des Vorgängers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PHASE 1: PROJEKTSTART, SPEZIFIKATION &amp; PREISKALKULATION (TAGE 0 BIS 19) — KRITISCHER PFAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="19" customHeight="1">
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 0</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>D: 2 T</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 2</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="n"/>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 2</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="n"/>
+      <c r="L11" s="16" t="inlineStr">
+        <is>
+          <t>D: 5 T</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="n"/>
+      <c r="N11" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 7</t>
+        </is>
+      </c>
+      <c r="O11" s="17" t="n"/>
+      <c r="R11" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 7</t>
+        </is>
+      </c>
+      <c r="S11" s="15" t="n"/>
+      <c r="T11" s="16" t="inlineStr">
+        <is>
+          <t>D: 5 T</t>
+        </is>
+      </c>
+      <c r="U11" s="15" t="n"/>
+      <c r="V11" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 12</t>
+        </is>
+      </c>
+      <c r="W11" s="17" t="n"/>
+      <c r="Z11" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 12</t>
+        </is>
+      </c>
+      <c r="AA11" s="15" t="n"/>
+      <c r="AB11" s="16" t="inlineStr">
+        <is>
+          <t>D: 3 T</t>
+        </is>
+      </c>
+      <c r="AC11" s="15" t="n"/>
+      <c r="AD11" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 15</t>
+        </is>
+      </c>
+      <c r="AE11" s="17" t="n"/>
+      <c r="AH11" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 15</t>
+        </is>
+      </c>
+      <c r="AI11" s="15" t="n"/>
+      <c r="AJ11" s="16" t="inlineStr">
+        <is>
+          <t>D: 4 T</t>
+        </is>
+      </c>
+      <c r="AK11" s="15" t="n"/>
+      <c r="AL11" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 19</t>
+        </is>
+      </c>
+      <c r="AM11" s="17" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>V1: Projektstart &amp; Kick-off
+[Jan Kluth]</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="20" t="n"/>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>V2: Anforderung &amp; Lastenheft
+[Mathias Vonau]</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="n"/>
+      <c r="L12" s="19" t="n"/>
+      <c r="M12" s="19" t="n"/>
+      <c r="N12" s="19" t="n"/>
+      <c r="O12" s="20" t="n"/>
+      <c r="P12" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="R12" s="18" t="inlineStr">
+        <is>
+          <t>V3: Marktrecherche Hardware
+[Marian Bolecke]</t>
+        </is>
+      </c>
+      <c r="S12" s="19" t="n"/>
+      <c r="T12" s="19" t="n"/>
+      <c r="U12" s="19" t="n"/>
+      <c r="V12" s="19" t="n"/>
+      <c r="W12" s="20" t="n"/>
+      <c r="X12" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="Z12" s="18" t="inlineStr">
+        <is>
+          <t>V4: Nutzwertanalyse (NWA)
+[Marian Bolecke]</t>
+        </is>
+      </c>
+      <c r="AA12" s="19" t="n"/>
+      <c r="AB12" s="19" t="n"/>
+      <c r="AC12" s="19" t="n"/>
+      <c r="AD12" s="19" t="n"/>
+      <c r="AE12" s="20" t="n"/>
+      <c r="AF12" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="AH12" s="18" t="inlineStr">
+        <is>
+          <t>V5: Angebot &amp; Kalkulation
+[Marian Bolecke]</t>
+        </is>
+      </c>
+      <c r="AI12" s="19" t="n"/>
+      <c r="AJ12" s="19" t="n"/>
+      <c r="AK12" s="19" t="n"/>
+      <c r="AL12" s="19" t="n"/>
+      <c r="AM12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="19" customHeight="1">
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 0</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n"/>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="n"/>
+      <c r="F13" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 2</t>
+        </is>
+      </c>
+      <c r="G13" s="26" t="n"/>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 2</t>
+        </is>
+      </c>
+      <c r="K13" s="23" t="n"/>
+      <c r="L13" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="M13" s="23" t="n"/>
+      <c r="N13" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 7</t>
+        </is>
+      </c>
+      <c r="O13" s="26" t="n"/>
+      <c r="R13" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 7</t>
+        </is>
+      </c>
+      <c r="S13" s="23" t="n"/>
+      <c r="T13" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="U13" s="23" t="n"/>
+      <c r="V13" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 12</t>
+        </is>
+      </c>
+      <c r="W13" s="26" t="n"/>
+      <c r="Z13" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 12</t>
+        </is>
+      </c>
+      <c r="AA13" s="23" t="n"/>
+      <c r="AB13" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="AC13" s="23" t="n"/>
+      <c r="AD13" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 15</t>
+        </is>
+      </c>
+      <c r="AE13" s="26" t="n"/>
+      <c r="AH13" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 15</t>
+        </is>
+      </c>
+      <c r="AI13" s="23" t="n"/>
+      <c r="AJ13" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="AK13" s="23" t="n"/>
+      <c r="AL13" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 19</t>
+        </is>
+      </c>
+      <c r="AM13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="14" customHeight="1"/>
+    <row r="15" ht="14" customHeight="1">
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │  (Angebotsabgabe &amp; Kundenentscheidung: Übergang von V5 nach V6 bei Tag 19)    ▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PHASE 2: BEAUFTRAGUNG, BESCHAFFUNG &amp; VORINSTALLATION / STAGING (TAGE 19 BIS 39) — KRITISCHER PFAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1">
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 19</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>D: 3 T</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 22</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="n"/>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 22</t>
+        </is>
+      </c>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>D: 10 T</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="n"/>
+      <c r="N17" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 32</t>
+        </is>
+      </c>
+      <c r="O17" s="17" t="n"/>
+      <c r="R17" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 32</t>
+        </is>
+      </c>
+      <c r="S17" s="15" t="n"/>
+      <c r="T17" s="16" t="inlineStr">
+        <is>
+          <t>D: 2 T</t>
+        </is>
+      </c>
+      <c r="U17" s="15" t="n"/>
+      <c r="V17" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 34</t>
+        </is>
+      </c>
+      <c r="W17" s="17" t="n"/>
+      <c r="Z17" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 34</t>
+        </is>
+      </c>
+      <c r="AA17" s="15" t="n"/>
+      <c r="AB17" s="16" t="inlineStr">
+        <is>
+          <t>D: 5 T</t>
+        </is>
+      </c>
+      <c r="AC17" s="15" t="n"/>
+      <c r="AD17" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 39</t>
+        </is>
+      </c>
+      <c r="AE17" s="17" t="n"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>V6: Kundenfreigabe / Auftrag
+[Jan Kluth]</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="20" t="n"/>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>V7: Bestellung &amp; Beschaffung
+[Marian Bolecke]</t>
+        </is>
+      </c>
+      <c r="K18" s="19" t="n"/>
+      <c r="L18" s="19" t="n"/>
+      <c r="M18" s="19" t="n"/>
+      <c r="N18" s="19" t="n"/>
+      <c r="O18" s="20" t="n"/>
+      <c r="P18" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="R18" s="18" t="inlineStr">
+        <is>
+          <t>V8: Prüfung nach § 377 HGB
+[Marco Schmidt]</t>
+        </is>
+      </c>
+      <c r="S18" s="19" t="n"/>
+      <c r="T18" s="19" t="n"/>
+      <c r="U18" s="19" t="n"/>
+      <c r="V18" s="19" t="n"/>
+      <c r="W18" s="20" t="n"/>
+      <c r="X18" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="Z18" s="18" t="inlineStr">
+        <is>
+          <t>V9: Vorinstallation &amp; Staging
+[Mathias &amp; Siyar]</t>
+        </is>
+      </c>
+      <c r="AA18" s="19" t="n"/>
+      <c r="AB18" s="19" t="n"/>
+      <c r="AC18" s="19" t="n"/>
+      <c r="AD18" s="19" t="n"/>
+      <c r="AE18" s="20" t="n"/>
+    </row>
+    <row r="19" ht="19" customHeight="1">
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 19</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n"/>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="n"/>
+      <c r="F19" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 22</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="n"/>
+      <c r="J19" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 22</t>
+        </is>
+      </c>
+      <c r="K19" s="23" t="n"/>
+      <c r="L19" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="M19" s="23" t="n"/>
+      <c r="N19" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 32</t>
+        </is>
+      </c>
+      <c r="O19" s="26" t="n"/>
+      <c r="R19" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 32</t>
+        </is>
+      </c>
+      <c r="S19" s="23" t="n"/>
+      <c r="T19" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="U19" s="23" t="n"/>
+      <c r="V19" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 34</t>
+        </is>
+      </c>
+      <c r="W19" s="26" t="n"/>
+      <c r="Z19" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 34</t>
+        </is>
+      </c>
+      <c r="AA19" s="23" t="n"/>
+      <c r="AB19" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="AC19" s="23" t="n"/>
+      <c r="AD19" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 39</t>
+        </is>
+      </c>
+      <c r="AE19" s="26" t="n"/>
+    </row>
+    <row r="20" ht="12" customHeight="1"/>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▼  VERZWEIGUNG NACH V9 (TAG 39): Vorgang V10 (Entsorgung) und Vorgang V11 (Montage) laufen PARALLEL!  ▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PHASE 3: PARALLELE VORGÄNGE (V10 || V11), GESAMTABNAHME &amp; PROJEKTABSCHLUSS (TAGE 39 BIS 46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="14" customHeight="1">
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>▲ PARALLELER ZWEIG A (Pufferzeit = 1 Tag):</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="19" customHeight="1">
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>FAZ: 39</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="n"/>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>D: 2 T</t>
+        </is>
+      </c>
+      <c r="E24" s="31" t="n"/>
+      <c r="F24" s="32" t="inlineStr">
+        <is>
+          <t>FEZ: 41</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="B25" s="34" t="inlineStr">
+        <is>
+          <t>V10: Entsorgung Altdrucker
+[Marco Schmidt]</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="35" t="n"/>
+      <c r="H25" s="36" t="inlineStr">
+        <is>
+          <t>➔ ↘</t>
+        </is>
+      </c>
+      <c r="J25" s="37" t="inlineStr">
+        <is>
+          <t>ZUSAMMENFÜHRUNG (V10 + V11):</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="19" customHeight="1">
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>SAZ: 40</t>
+        </is>
+      </c>
+      <c r="C26" s="39" t="n"/>
+      <c r="D26" s="40" t="inlineStr">
+        <is>
+          <t>GP: 1 T</t>
+        </is>
+      </c>
+      <c r="E26" s="39" t="n"/>
+      <c r="F26" s="41" t="inlineStr">
+        <is>
+          <t>SEZ: 42</t>
+        </is>
+      </c>
+      <c r="G26" s="42" t="n"/>
+      <c r="J26" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 42</t>
+        </is>
+      </c>
+      <c r="K26" s="15" t="n"/>
+      <c r="L26" s="16" t="inlineStr">
+        <is>
+          <t>D: 2 T</t>
+        </is>
+      </c>
+      <c r="M26" s="15" t="n"/>
+      <c r="N26" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 44</t>
+        </is>
+      </c>
+      <c r="O26" s="17" t="n"/>
+      <c r="R26" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 44</t>
+        </is>
+      </c>
+      <c r="S26" s="15" t="n"/>
+      <c r="T26" s="16" t="inlineStr">
+        <is>
+          <t>D: 1 T</t>
+        </is>
+      </c>
+      <c r="U26" s="15" t="n"/>
+      <c r="V26" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 45</t>
+        </is>
+      </c>
+      <c r="W26" s="17" t="n"/>
+      <c r="Z26" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 45</t>
+        </is>
+      </c>
+      <c r="AA26" s="15" t="n"/>
+      <c r="AB26" s="16" t="inlineStr">
+        <is>
+          <t>D: 1 T</t>
+        </is>
+      </c>
+      <c r="AC26" s="15" t="n"/>
+      <c r="AD26" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 46</t>
+        </is>
+      </c>
+      <c r="AE26" s="17" t="n"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="J27" s="18" t="inlineStr">
+        <is>
+          <t>V12: Funktionstest &amp; Abnahme
+[Gesamtes Team]</t>
+        </is>
+      </c>
+      <c r="K27" s="19" t="n"/>
+      <c r="L27" s="19" t="n"/>
+      <c r="M27" s="19" t="n"/>
+      <c r="N27" s="19" t="n"/>
+      <c r="O27" s="20" t="n"/>
+      <c r="P27" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="R27" s="18" t="inlineStr">
+        <is>
+          <t>V13: Übergabe &amp; Dokumentation
+[Jan Kluth]</t>
+        </is>
+      </c>
+      <c r="S27" s="19" t="n"/>
+      <c r="T27" s="19" t="n"/>
+      <c r="U27" s="19" t="n"/>
+      <c r="V27" s="19" t="n"/>
+      <c r="W27" s="20" t="n"/>
+      <c r="X27" s="21" t="inlineStr">
+        <is>
+          <t>➔</t>
+        </is>
+      </c>
+      <c r="Z27" s="18" t="inlineStr">
+        <is>
+          <t>V14: Lessons Learned &amp; Abschluss
+[Gesamtes Team]</t>
+        </is>
+      </c>
+      <c r="AA27" s="19" t="n"/>
+      <c r="AB27" s="19" t="n"/>
+      <c r="AC27" s="19" t="n"/>
+      <c r="AD27" s="19" t="n"/>
+      <c r="AE27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="19" customHeight="1">
+      <c r="B28" s="43" t="inlineStr">
+        <is>
+          <t>▼ PARALLELER ZWEIG B (Kritischer Pfad):</t>
+        </is>
+      </c>
+      <c r="J28" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 42</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="n"/>
+      <c r="L28" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="M28" s="23" t="n"/>
+      <c r="N28" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 44</t>
+        </is>
+      </c>
+      <c r="O28" s="26" t="n"/>
+      <c r="R28" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 44</t>
+        </is>
+      </c>
+      <c r="S28" s="23" t="n"/>
+      <c r="T28" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="U28" s="23" t="n"/>
+      <c r="V28" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 45</t>
+        </is>
+      </c>
+      <c r="W28" s="26" t="n"/>
+      <c r="Z28" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 45</t>
+        </is>
+      </c>
+      <c r="AA28" s="23" t="n"/>
+      <c r="AB28" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="AC28" s="23" t="n"/>
+      <c r="AD28" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 46</t>
+        </is>
+      </c>
+      <c r="AE28" s="26" t="n"/>
+    </row>
+    <row r="29" ht="19" customHeight="1">
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 39</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>D: 3 T</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 42</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="n"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>V11: Lieferung &amp; Montage vor Ort
+[Mathias &amp; Siyar]</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="20" t="n"/>
+      <c r="H30" s="44" t="inlineStr">
+        <is>
+          <t>➔ ↗</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1">
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>SAZ: 39</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="n"/>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>GP: 0</t>
+        </is>
+      </c>
+      <c r="E31" s="23" t="n"/>
+      <c r="F31" s="25" t="inlineStr">
+        <is>
+          <t>SEZ: 42</t>
+        </is>
+      </c>
+      <c r="G31" s="26" t="n"/>
+    </row>
+    <row r="33" ht="12" customHeight="1"/>
+    <row r="34" ht="28" customHeight="1">
+      <c r="B34" s="45" t="inlineStr">
+        <is>
+          <t>KRITISCHER PFAD (ROT): V1 ➔ V2 ➔ V3 ➔ V4 ➔ V5 ➔ V6 ➔ V7 ➔ V8 ➔ V9 ➔ V11 ➔ V12 ➔ V13 ➔ V14  |  GESAMTDAUER: 46 ARBEITSTAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="B35" s="46" t="inlineStr">
+        <is>
+          <t>Parallele Ausführung: V10 (Entsorgung Altdrucker) besitzt 1 Tag Gesamtpuffer (GP = 1, FP = 1) und beeinflusst das Projektende nicht, solange die Dauer ≤ 3 Tage bleibt.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="133">
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="AD17:AE17"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="V17:W17"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="Z11:AA11"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="L6:AM6"/>
+    <mergeCell ref="V28:W28"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B21:AM21"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="AF12:AG12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="Z13:AA13"/>
+    <mergeCell ref="AD26:AE26"/>
+    <mergeCell ref="AB13:AC13"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="L8:AM8"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="AH13:AI13"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="R12:W12"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="V19:W19"/>
+    <mergeCell ref="B22:AM22"/>
+    <mergeCell ref="AD28:AE28"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="R18:W18"/>
+    <mergeCell ref="V11:W11"/>
+    <mergeCell ref="J18:O18"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="AH11:AI11"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B7:J7"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="Z27:AE27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="J27:O27"/>
+    <mergeCell ref="B35:AM35"/>
+    <mergeCell ref="Z12:AE12"/>
+    <mergeCell ref="V13:W13"/>
+    <mergeCell ref="Z26:AA26"/>
+    <mergeCell ref="AB26:AC26"/>
+    <mergeCell ref="B16:AM16"/>
+    <mergeCell ref="B3:AM3"/>
+    <mergeCell ref="AD19:AE19"/>
+    <mergeCell ref="P27:Q27"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="B2:AM2"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="B5:J5"/>
+    <mergeCell ref="Z17:AA17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="AB11:AC11"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="AD11:AE11"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="T17:U17"/>
+    <mergeCell ref="B34:AM34"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="Z28:AA28"/>
+    <mergeCell ref="T19:U19"/>
+    <mergeCell ref="AB28:AC28"/>
+    <mergeCell ref="L5:AM5"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="T28:U28"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="B15:AM15"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="X12:Y12"/>
+    <mergeCell ref="R11:S11"/>
+    <mergeCell ref="AJ11:AK11"/>
+    <mergeCell ref="R27:W27"/>
+    <mergeCell ref="AL11:AM11"/>
+    <mergeCell ref="Z18:AE18"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="AD13:AE13"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="J25:O25"/>
+    <mergeCell ref="AJ13:AK13"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="AL13:AM13"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="L7:AM7"/>
+    <mergeCell ref="T26:U26"/>
+    <mergeCell ref="V26:W26"/>
+    <mergeCell ref="T13:U13"/>
+    <mergeCell ref="AB17:AC17"/>
+    <mergeCell ref="AH12:AM12"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="B10:AM10"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="Z19:AA19"/>
+    <mergeCell ref="AB19:AC19"/>
+    <mergeCell ref="X27:Y27"/>
+    <mergeCell ref="J17:K17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -655,754 +2178,754 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>Vorgangsknoten-Berechnungstabelle nach DIN 69900 (Knotenvorgangsmodell CPM)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Vorgangs-Nr.</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="48" t="inlineStr">
         <is>
           <t>Vorgangsbezeichnung</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="48" t="inlineStr">
         <is>
           <t>Dauer (Tage)</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Vorgaenger</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="D3" s="48" t="inlineStr">
+        <is>
+          <t>Vorgänger</t>
+        </is>
+      </c>
+      <c r="E3" s="48" t="inlineStr">
         <is>
           <t>Nachfolger</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>FAZ (Fruehester Anfang)</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>FEZ (Fruehestes Ende)</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>SAZ (Spaetester Anfang)</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>SEZ (Spaetestes Ende)</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="F3" s="48" t="inlineStr">
+        <is>
+          <t>FAZ (Frühester Anfang)</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="inlineStr">
+        <is>
+          <t>FEZ (Frühestes Ende)</t>
+        </is>
+      </c>
+      <c r="H3" s="48" t="inlineStr">
+        <is>
+          <t>SAZ (Spätester Anfang)</t>
+        </is>
+      </c>
+      <c r="I3" s="48" t="inlineStr">
+        <is>
+          <t>SEZ (Spätestes Ende)</t>
+        </is>
+      </c>
+      <c r="J3" s="48" t="inlineStr">
         <is>
           <t>Gesamtpuffer (GP)</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>Kritisch?</t>
+      <c r="K3" s="48" t="inlineStr">
+        <is>
+          <t>Kritisch / Status</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="49" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="50" t="inlineStr">
         <is>
           <t>Projektstart &amp; Kick-off-Meeting</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="51" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="F4" s="9" t="n">
+      <c r="F4" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="9" t="n">
+      <c r="G4" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="9" t="n">
+      <c r="H4" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="9" t="n">
+      <c r="I4" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="J4" s="10" t="n">
+      <c r="J4" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K4" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="49" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="50" t="inlineStr">
         <is>
           <t>Anforderungsanalyse &amp; Lastenhefterstellung</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="49" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="51" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="H5" s="9" t="n">
+      <c r="H5" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I5" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="J5" s="10" t="n">
+      <c r="J5" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K5" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="49" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="50" t="inlineStr">
         <is>
           <t>Marktrecherche &amp; Einholen von Angeboten</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="49" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="51" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="51" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="51" t="n">
         <v>12</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="51" t="n">
         <v>12</v>
       </c>
-      <c r="J6" s="10" t="n">
+      <c r="J6" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="7" t="inlineStr">
+      <c r="K6" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>Nutzwertanalyse (Hardware-Auswahl)</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="51" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="51" t="inlineStr">
         <is>
           <t>V5</t>
         </is>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="51" t="n">
         <v>12</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="51" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="H7" s="51" t="n">
         <v>12</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="I7" s="51" t="n">
         <v>15</v>
       </c>
-      <c r="J7" s="10" t="n">
+      <c r="J7" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="K7" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>V5</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Angebotserstellung &amp; Vorwaertskalkulation</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="n">
+      <c r="B8" s="50" t="inlineStr">
+        <is>
+          <t>Angebotserstellung &amp; Vorwärtskalkulation</t>
+        </is>
+      </c>
+      <c r="C8" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="51" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="51" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="51" t="n">
         <v>15</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="51" t="n">
         <v>19</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="H8" s="51" t="n">
         <v>15</v>
       </c>
-      <c r="I8" s="9" t="n">
+      <c r="I8" s="51" t="n">
         <v>19</v>
       </c>
-      <c r="J8" s="10" t="n">
+      <c r="J8" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="7" t="inlineStr">
+      <c r="K8" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="49" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="50" t="inlineStr">
         <is>
           <t>Kundenfreigabe &amp; Auftragsvergabe</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="51" t="inlineStr">
         <is>
           <t>V5</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="51" t="inlineStr">
         <is>
           <t>V7</t>
         </is>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="51" t="n">
         <v>19</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="51" t="n">
         <v>22</v>
       </c>
-      <c r="H9" s="9" t="n">
+      <c r="H9" s="51" t="n">
         <v>19</v>
       </c>
-      <c r="I9" s="9" t="n">
+      <c r="I9" s="51" t="n">
         <v>22</v>
       </c>
-      <c r="J9" s="10" t="n">
+      <c r="J9" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K9" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t>V7</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="50" t="inlineStr">
         <is>
           <t>Bestellung &amp; Beschaffung der Komponenten</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="49" t="n">
         <v>10</v>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="51" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="51" t="inlineStr">
         <is>
           <t>V8</t>
         </is>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="51" t="n">
         <v>22</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="51" t="n">
         <v>32</v>
       </c>
-      <c r="H10" s="9" t="n">
+      <c r="H10" s="51" t="n">
         <v>22</v>
       </c>
-      <c r="I10" s="9" t="n">
+      <c r="I10" s="51" t="n">
         <v>32</v>
       </c>
-      <c r="J10" s="10" t="n">
+      <c r="J10" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="7" t="inlineStr">
+      <c r="K10" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="49" t="inlineStr">
         <is>
           <t>V8</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Wareneingangspruefung nach Paragraph 377 HGB</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
+      <c r="B11" s="50" t="inlineStr">
+        <is>
+          <t>Wareneingangsprüfung nach § 377 HGB</t>
+        </is>
+      </c>
+      <c r="C11" s="49" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="51" t="inlineStr">
         <is>
           <t>V7</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="51" t="inlineStr">
         <is>
           <t>V9</t>
         </is>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="51" t="n">
         <v>32</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G11" s="51" t="n">
         <v>34</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H11" s="51" t="n">
         <v>32</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I11" s="51" t="n">
         <v>34</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="J11" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="K11" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>V9</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="50" t="inlineStr">
         <is>
           <t>Vorinstallation, Konfiguration &amp; Staging</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="49" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="51" t="inlineStr">
         <is>
           <t>V8</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="51" t="inlineStr">
         <is>
           <t>V10, V11</t>
         </is>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F12" s="51" t="n">
         <v>34</v>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G12" s="51" t="n">
         <v>39</v>
       </c>
-      <c r="H12" s="9" t="n">
+      <c r="H12" s="51" t="n">
         <v>34</v>
       </c>
-      <c r="I12" s="9" t="n">
+      <c r="I12" s="51" t="n">
         <v>39</v>
       </c>
-      <c r="J12" s="10" t="n">
+      <c r="J12" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="7" t="inlineStr">
+      <c r="K12" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="53" t="inlineStr">
         <is>
           <t>V10</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="54" t="inlineStr">
         <is>
           <t>Fachgerechte Entsorgung Altdrucker (ElektroG)</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="55" t="inlineStr">
         <is>
           <t>V9</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="55" t="inlineStr">
         <is>
           <t>V12</t>
         </is>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="55" t="n">
         <v>39</v>
       </c>
-      <c r="G13" s="13" t="n">
+      <c r="G13" s="55" t="n">
         <v>41</v>
       </c>
-      <c r="H13" s="13" t="n">
+      <c r="H13" s="55" t="n">
         <v>40</v>
       </c>
-      <c r="I13" s="13" t="n">
+      <c r="I13" s="55" t="n">
         <v>42</v>
       </c>
-      <c r="J13" s="14" t="n">
+      <c r="J13" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>Nein (1 Tag Puffer)</t>
+      <c r="K13" s="53" t="inlineStr">
+        <is>
+          <t>NEIN (1 Tag Puffer, parallel zu V11)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="49" t="inlineStr">
         <is>
           <t>V11</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="50" t="inlineStr">
         <is>
           <t>Lieferung, Montage &amp; Verkabelung vor Ort</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="51" t="inlineStr">
         <is>
           <t>V9</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="51" t="inlineStr">
         <is>
           <t>V12</t>
         </is>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F14" s="51" t="n">
         <v>39</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="51" t="n">
         <v>42</v>
       </c>
-      <c r="H14" s="9" t="n">
+      <c r="H14" s="51" t="n">
         <v>39</v>
       </c>
-      <c r="I14" s="9" t="n">
+      <c r="I14" s="51" t="n">
         <v>42</v>
       </c>
-      <c r="J14" s="10" t="n">
+      <c r="J14" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="K14" s="49" t="inlineStr">
+        <is>
+          <t>JA (Kritischer Pfad, parallel zu V10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>V12</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>Funktionstest &amp; Gesamtabnahme</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="51" t="inlineStr">
+        <is>
+          <t>V10, V11</t>
+        </is>
+      </c>
+      <c r="E15" s="51" t="inlineStr">
+        <is>
+          <t>V13</t>
+        </is>
+      </c>
+      <c r="F15" s="51" t="n">
+        <v>42</v>
+      </c>
+      <c r="G15" s="51" t="n">
+        <v>44</v>
+      </c>
+      <c r="H15" s="51" t="n">
+        <v>42</v>
+      </c>
+      <c r="I15" s="51" t="n">
+        <v>44</v>
+      </c>
+      <c r="J15" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>V13</t>
+        </is>
+      </c>
+      <c r="B16" s="50" t="inlineStr">
+        <is>
+          <t>Mitarbeitereinweisung &amp; formelle Übergabe</t>
+        </is>
+      </c>
+      <c r="C16" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="51" t="inlineStr">
         <is>
           <t>V12</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Funktionstest &amp; Gesamtabnahme</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>V10, V11</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E16" s="51" t="inlineStr">
+        <is>
+          <t>V14</t>
+        </is>
+      </c>
+      <c r="F16" s="51" t="n">
+        <v>44</v>
+      </c>
+      <c r="G16" s="51" t="n">
+        <v>45</v>
+      </c>
+      <c r="H16" s="51" t="n">
+        <v>44</v>
+      </c>
+      <c r="I16" s="51" t="n">
+        <v>45</v>
+      </c>
+      <c r="J16" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="49" t="inlineStr">
+        <is>
+          <t>JA (Kritischer Pfad)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>V14</t>
+        </is>
+      </c>
+      <c r="B17" s="50" t="inlineStr">
+        <is>
+          <t>Projektabschlussbericht &amp; Lessons Learned</t>
+        </is>
+      </c>
+      <c r="C17" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="51" t="inlineStr">
         <is>
           <t>V13</t>
         </is>
       </c>
-      <c r="F15" s="9" t="n">
-        <v>42</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="H15" s="9" t="n">
-        <v>42</v>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="J15" s="10" t="n">
+      <c r="E17" s="51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="51" t="n">
+        <v>45</v>
+      </c>
+      <c r="G17" s="51" t="n">
+        <v>46</v>
+      </c>
+      <c r="H17" s="51" t="n">
+        <v>45</v>
+      </c>
+      <c r="I17" s="51" t="n">
+        <v>46</v>
+      </c>
+      <c r="J17" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K17" s="49" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>V13</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Mitarbeitereinweisung &amp; formelle Uebergabe</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>V12</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>V14</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="I16" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="J16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="7" t="inlineStr">
-        <is>
-          <t>JA (Kritischer Pfad)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>V14</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Projektabschlussbericht &amp; Lessons Learned</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>V13</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>46</v>
-      </c>
-      <c r="H17" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="I17" s="9" t="n">
-        <v>46</v>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="7" t="inlineStr">
-        <is>
-          <t>JA (Kritischer Pfad)</t>
-        </is>
-      </c>
-    </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="57" t="inlineStr">
         <is>
           <t>Gesamte Projektdauer auf dem kritischen Pfad:</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>46 Arbeitstage (Pufferzeit im Gesamtprojekt: 0 Tage auf krit. Pfad / 1 Tag bei V10)</t>
+      <c r="F19" s="58" t="inlineStr">
+        <is>
+          <t>46 Arbeitstage (Gesamtpuffer auf kritischem Pfad: 0 Tage | Puffer bei V10: 1 Tag)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="59" t="inlineStr">
         <is>
           <t>Formeln &amp; Rechenregeln der Netzplantechnik nach DIN 69900:</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>1. Vorwaertsrechnung: FEZ = FAZ + Dauer. Bei mehreren Vorgaengern gilt fuer den Nachfolger: FAZ = Maximum aller FEZ der Vorgaenger.</t>
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>1. Vorwärtsrechnung: FEZ = FAZ + Dauer. Bei mehreren Vorgängern gilt für den Nachfolger: FAZ = Maximum aller FEZ der Vorgänger.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>2. Rueckwaertsrechnung: SAZ = SEZ - Dauer. Bei mehreren Nachfolgern gilt fuer den Vorgaenger: SEZ = Minimum aller SAZ der Nachfolger.</t>
+      <c r="A23" s="60" t="inlineStr">
+        <is>
+          <t>2. Rückwärtsrechnung: SAZ = SEZ - Dauer. Bei mehreren Nachfolgern gilt für den Vorgänger: SEZ = Minimum aller SAZ der Nachfolger.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr">
         <is>
           <t>3. Gesamtpuffer (GP): GP = SAZ - FAZ = SEZ - FEZ. Ein Vorgang mit GP = 0 liegt zwingend auf dem kritischen Pfad!</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>4. Freier Puffer (FP): FP = min(FAZ_Nachfolger) - FEZ. Gibt an, um wie viel ein Vorgang verzoegert werden kann, ohne den FAZ des Nachfolgers zu beeinflussen.</t>
+      <c r="A25" s="60" t="inlineStr">
+        <is>
+          <t>4. Freier Puffer (FP): FP = min(FAZ_Nachfolger) - FEZ. Gibt an, um wie viel ein Vorgang verzögert werden kann, ohne den FAZ des Nachfolgers zu beeinflussen.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>5. Kritischer Pfad: Kette der Vorgaenge von Projektstart bis Projektende ohne Puffer (GP = 0). Jede Verzoegerung verlaengert das Gesamtprojekt!</t>
+      <c r="A26" s="60" t="inlineStr">
+        <is>
+          <t>5. Parallele Vorgänge: V10 (Entsorgung) und V11 (Montage) starten beide nach V9 (FAZ = 39). V11 bestimmt den kritischen Pfad (D=3, FEZ=42). V10 (D=2, FEZ=41) besitzt 1 Tag Puffer (GP=1, FP=1).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Netzplan: Saemtliche Text-Hinweise bei Verzweigungen und Zusammenfuehrungen entfernt, reine Pfeil- und Verbindungslinien-Fuehrung
</commit_message>
<xml_diff>
--- a/docs/01_Projektorganisation/Netzplan.xlsx
+++ b/docs/01_Projektorganisation/Netzplan.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -127,8 +127,20 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="002F5597"/>
-      <sz val="8.5"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -139,20 +151,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002F5597"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F497D"/>
-      <sz val="8.5"/>
+      <color rgb="002F5597"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -162,54 +168,54 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5597"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00404040"/>
       <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002F5597"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F497D"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="009C0006"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="11">
@@ -241,17 +247,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -265,7 +271,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -414,6 +420,11 @@
       </bottom>
     </border>
     <border>
+      <top style="medium">
+        <color rgb="00C00000"/>
+      </top>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="00D9D9D9"/>
       </left>
@@ -595,54 +606,52 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -678,11 +687,11 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1048,42 +1057,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AM35"/>
+  <dimension ref="B2:AM33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6.2" customWidth="1" min="1" max="1"/>
+    <col width="3.8" customWidth="1" min="1" max="1"/>
     <col width="6.2" customWidth="1" min="2" max="2"/>
     <col width="6.2" customWidth="1" min="3" max="3"/>
     <col width="6.2" customWidth="1" min="4" max="4"/>
     <col width="6.2" customWidth="1" min="5" max="5"/>
     <col width="6.2" customWidth="1" min="6" max="6"/>
     <col width="6.2" customWidth="1" min="7" max="7"/>
-    <col width="4" customWidth="1" min="8" max="8"/>
-    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="3.8" customWidth="1" min="8" max="8"/>
+    <col width="3.8" customWidth="1" min="9" max="9"/>
     <col width="6.2" customWidth="1" min="10" max="10"/>
     <col width="6.2" customWidth="1" min="11" max="11"/>
     <col width="6.2" customWidth="1" min="12" max="12"/>
     <col width="6.2" customWidth="1" min="13" max="13"/>
     <col width="6.2" customWidth="1" min="14" max="14"/>
     <col width="6.2" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
-    <col width="4" customWidth="1" min="17" max="17"/>
+    <col width="3.8" customWidth="1" min="16" max="16"/>
+    <col width="3.8" customWidth="1" min="17" max="17"/>
     <col width="6.2" customWidth="1" min="18" max="18"/>
     <col width="6.2" customWidth="1" min="19" max="19"/>
     <col width="6.2" customWidth="1" min="20" max="20"/>
     <col width="6.2" customWidth="1" min="21" max="21"/>
     <col width="6.2" customWidth="1" min="22" max="22"/>
     <col width="6.2" customWidth="1" min="23" max="23"/>
-    <col width="4" customWidth="1" min="24" max="24"/>
-    <col width="4" customWidth="1" min="25" max="25"/>
+    <col width="3.8" customWidth="1" min="24" max="24"/>
+    <col width="3.8" customWidth="1" min="25" max="25"/>
     <col width="6.2" customWidth="1" min="26" max="26"/>
     <col width="6.2" customWidth="1" min="27" max="27"/>
     <col width="6.2" customWidth="1" min="28" max="28"/>
     <col width="6.2" customWidth="1" min="29" max="29"/>
     <col width="6.2" customWidth="1" min="30" max="30"/>
     <col width="6.2" customWidth="1" min="31" max="31"/>
-    <col width="4" customWidth="1" min="32" max="32"/>
-    <col width="4" customWidth="1" min="33" max="33"/>
+    <col width="3.8" customWidth="1" min="32" max="32"/>
+    <col width="3.8" customWidth="1" min="33" max="33"/>
     <col width="6.2" customWidth="1" min="34" max="34"/>
     <col width="6.2" customWidth="1" min="35" max="35"/>
     <col width="6.2" customWidth="1" min="36" max="36"/>
@@ -1112,7 +1121,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="10" customHeight="1"/>
+    <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -1129,7 +1138,7 @@
       <c r="J5" s="4" t="n"/>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Erläuterung der Pfade &amp; Farben im Netzplan:</t>
+          <t>Pfade &amp; Farben:</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1166,7 @@
       <c r="J6" s="4" t="n"/>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>■ KRITISCHER PFAD (Rot / Warmgelb): Gesamtpuffer GP = 0. Jede Verzögerung verschiebt unmittelbar das Projektende (Dauer: 46 Arbeitstage).</t>
+          <t>■ KRITISCHER PFAD (Rot / Warmgelb): Gesamtpuffer GP = 0 (Verzögerung verschiebt Projektende).</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1186,7 @@
       <c r="J7" s="4" t="n"/>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>■ PARALLELE VORGÄNGE &amp; PUFFER (Blau): V10 (Entsorgung Altdrucker) läuft parallel zu V11 (Montage). V10 hat 1 Tag Gesamtpuffer (GP = 1).</t>
+          <t>■ PARALLELER VORGANG MIT PUFFER (Blau): V10 (Entsorgung Altdrucker) läuft parallel zu V11 und hat GP = 1 Tag Puffer.</t>
         </is>
       </c>
     </row>
@@ -1205,14 +1214,14 @@
       <c r="J8" s="4" t="n"/>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>➔ Normalfolge (Ende-Anfang EA = 0): Der Nachfolger beginnt frühestens unmittelbar nach Beendigung des Vorgängers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
+          <t>➔ Normalfolge (Ende-Anfang EA = 0): Nachfolger beginnt nach Ende des Vorgängers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PHASE 1: PROJEKTSTART, SPEZIFIKATION &amp; PREISKALKULATION (TAGE 0 BIS 19) — KRITISCHER PFAD</t>
+          <t xml:space="preserve">  PHASE 1: PROJEKTSTART, SPEZIFIKATION &amp; PREISKALKULATION (TAGE 0 BIS 19)</t>
         </is>
       </c>
     </row>
@@ -1477,18 +1486,56 @@
       </c>
       <c r="AM13" s="26" t="n"/>
     </row>
-    <row r="14" ht="14" customHeight="1"/>
-    <row r="15" ht="14" customHeight="1">
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │  (Angebotsabgabe &amp; Kundenentscheidung: Übergang von V5 nach V6 bei Tag 19)    ▼</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
+    <row r="14" ht="12" customHeight="1">
+      <c r="AK14" s="27" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="12" customHeight="1">
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="n"/>
+      <c r="G15" s="29" t="n"/>
+      <c r="H15" s="29" t="n"/>
+      <c r="I15" s="29" t="n"/>
+      <c r="J15" s="29" t="n"/>
+      <c r="K15" s="29" t="n"/>
+      <c r="L15" s="29" t="n"/>
+      <c r="M15" s="29" t="n"/>
+      <c r="N15" s="29" t="n"/>
+      <c r="O15" s="29" t="n"/>
+      <c r="P15" s="29" t="n"/>
+      <c r="Q15" s="29" t="n"/>
+      <c r="R15" s="29" t="n"/>
+      <c r="S15" s="29" t="n"/>
+      <c r="T15" s="29" t="n"/>
+      <c r="U15" s="29" t="n"/>
+      <c r="V15" s="29" t="n"/>
+      <c r="W15" s="29" t="n"/>
+      <c r="X15" s="29" t="n"/>
+      <c r="Y15" s="29" t="n"/>
+      <c r="Z15" s="29" t="n"/>
+      <c r="AA15" s="29" t="n"/>
+      <c r="AB15" s="29" t="n"/>
+      <c r="AC15" s="29" t="n"/>
+      <c r="AD15" s="29" t="n"/>
+      <c r="AE15" s="29" t="n"/>
+      <c r="AF15" s="29" t="n"/>
+      <c r="AG15" s="29" t="n"/>
+      <c r="AH15" s="29" t="n"/>
+      <c r="AI15" s="29" t="n"/>
+      <c r="AJ15" s="29" t="n"/>
+      <c r="AK15" s="29" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PHASE 2: BEAUFTRAGUNG, BESCHAFFUNG &amp; VORINSTALLATION / STAGING (TAGE 19 BIS 39) — KRITISCHER PFAD</t>
+          <t xml:space="preserve">  PHASE 2: BEAUFTRAGUNG, BESCHAFFUNG &amp; VORINSTALLATION / STAGING (TAGE 19 BIS 39)</t>
         </is>
       </c>
     </row>
@@ -1701,50 +1748,80 @@
       </c>
       <c r="AE19" s="26" t="n"/>
     </row>
-    <row r="20" ht="12" customHeight="1"/>
-    <row r="21" ht="18" customHeight="1">
-      <c r="B21" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▼  VERZWEIGUNG NACH V9 (TAG 39): Vorgang V10 (Entsorgung) und Vorgang V11 (Montage) laufen PARALLEL!  ▼</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
+    <row r="20" ht="12" customHeight="1">
+      <c r="AC20" s="27" t="inlineStr">
+        <is>
+          <t>│</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="12" customHeight="1">
+      <c r="E21" s="28" t="inlineStr">
+        <is>
+          <t>▼</t>
+        </is>
+      </c>
+      <c r="F21" s="29" t="n"/>
+      <c r="G21" s="29" t="n"/>
+      <c r="H21" s="29" t="n"/>
+      <c r="I21" s="29" t="n"/>
+      <c r="J21" s="29" t="n"/>
+      <c r="K21" s="29" t="n"/>
+      <c r="L21" s="29" t="n"/>
+      <c r="M21" s="29" t="n"/>
+      <c r="N21" s="29" t="n"/>
+      <c r="O21" s="29" t="n"/>
+      <c r="P21" s="29" t="n"/>
+      <c r="Q21" s="29" t="n"/>
+      <c r="R21" s="29" t="n"/>
+      <c r="S21" s="29" t="n"/>
+      <c r="T21" s="29" t="n"/>
+      <c r="U21" s="29" t="n"/>
+      <c r="V21" s="29" t="n"/>
+      <c r="W21" s="29" t="n"/>
+      <c r="X21" s="29" t="n"/>
+      <c r="Y21" s="29" t="n"/>
+      <c r="Z21" s="29" t="n"/>
+      <c r="AA21" s="29" t="n"/>
+      <c r="AB21" s="29" t="n"/>
+      <c r="AC21" s="29" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PHASE 3: PARALLELE VORGÄNGE (V10 || V11), GESAMTABNAHME &amp; PROJEKTABSCHLUSS (TAGE 39 BIS 46)</t>
+          <t xml:space="preserve">  PHASE 3: PARALLELE AUSFÜHRUNG (V10 || V11), ROLLOUT &amp; ABSCHLUSS (TAGE 39 BIS 46)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="14" customHeight="1">
-      <c r="B23" s="29" t="inlineStr">
-        <is>
-          <t>▲ PARALLELER ZWEIG A (Pufferzeit = 1 Tag):</t>
+      <c r="E23" s="30" t="inlineStr">
+        <is>
+          <t>▼</t>
         </is>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="B24" s="30" t="inlineStr">
+      <c r="B24" s="31" t="inlineStr">
         <is>
           <t>FAZ: 39</t>
         </is>
       </c>
-      <c r="C24" s="31" t="n"/>
-      <c r="D24" s="32" t="inlineStr">
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="33" t="inlineStr">
         <is>
           <t>D: 2 T</t>
         </is>
       </c>
-      <c r="E24" s="31" t="n"/>
-      <c r="F24" s="32" t="inlineStr">
+      <c r="E24" s="32" t="n"/>
+      <c r="F24" s="33" t="inlineStr">
         <is>
           <t>FEZ: 41</t>
         </is>
       </c>
-      <c r="G24" s="33" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="34" t="inlineStr">
+      <c r="G24" s="34" t="n"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t>V10: Entsorgung Altdrucker
 [Marco Schmidt]</t>
@@ -1754,15 +1831,10 @@
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="35" t="n"/>
-      <c r="H25" s="36" t="inlineStr">
+      <c r="G25" s="36" t="n"/>
+      <c r="H25" s="37" t="inlineStr">
         <is>
           <t>➔ ↘</t>
-        </is>
-      </c>
-      <c r="J25" s="37" t="inlineStr">
-        <is>
-          <t>ZUSAMMENFÜHRUNG (V10 + V11):</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1912,17 @@
       </c>
       <c r="AE26" s="17" t="n"/>
     </row>
-    <row r="27" ht="32" customHeight="1">
+    <row r="27" ht="16" customHeight="1">
+      <c r="E27" s="43" t="inlineStr">
+        <is>
+          <t>│  ▼</t>
+        </is>
+      </c>
+      <c r="I27" s="44" t="inlineStr">
+        <is>
+          <t>►</t>
+        </is>
+      </c>
       <c r="J27" s="18" t="inlineStr">
         <is>
           <t>V12: Funktionstest &amp; Abnahme
@@ -1886,11 +1968,24 @@
       <c r="AE27" s="20" t="n"/>
     </row>
     <row r="28" ht="19" customHeight="1">
-      <c r="B28" s="43" t="inlineStr">
-        <is>
-          <t>▼ PARALLELER ZWEIG B (Kritischer Pfad):</t>
-        </is>
-      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>FAZ: 39</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>D: 3 T</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>FEZ: 42</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="n"/>
       <c r="J28" s="22" t="inlineStr">
         <is>
           <t>SAZ: 42</t>
@@ -1946,98 +2041,67 @@
       </c>
       <c r="AE28" s="26" t="n"/>
     </row>
-    <row r="29" ht="19" customHeight="1">
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>FAZ: 39</t>
-        </is>
-      </c>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="16" t="inlineStr">
-        <is>
-          <t>D: 3 T</t>
-        </is>
-      </c>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="16" t="inlineStr">
-        <is>
-          <t>FEZ: 42</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="n"/>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="B30" s="18" t="inlineStr">
+    <row r="29" ht="32" customHeight="1">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>V11: Lieferung &amp; Montage vor Ort
 [Mathias &amp; Siyar]</t>
         </is>
       </c>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="19" t="n"/>
-      <c r="E30" s="19" t="n"/>
-      <c r="F30" s="19" t="n"/>
-      <c r="G30" s="20" t="n"/>
-      <c r="H30" s="44" t="inlineStr">
+      <c r="C29" s="19" t="n"/>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="20" t="n"/>
+      <c r="H29" s="45" t="inlineStr">
         <is>
           <t>➔ ↗</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
-      <c r="B31" s="22" t="inlineStr">
+    <row r="30" ht="19" customHeight="1">
+      <c r="B30" s="22" t="inlineStr">
         <is>
           <t>SAZ: 39</t>
         </is>
       </c>
-      <c r="C31" s="23" t="n"/>
-      <c r="D31" s="24" t="inlineStr">
+      <c r="C30" s="23" t="n"/>
+      <c r="D30" s="24" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="E31" s="23" t="n"/>
-      <c r="F31" s="25" t="inlineStr">
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="25" t="inlineStr">
         <is>
           <t>SEZ: 42</t>
         </is>
       </c>
-      <c r="G31" s="26" t="n"/>
-    </row>
-    <row r="33" ht="12" customHeight="1"/>
-    <row r="34" ht="28" customHeight="1">
-      <c r="B34" s="45" t="inlineStr">
+      <c r="G30" s="26" t="n"/>
+    </row>
+    <row r="32" ht="10" customHeight="1"/>
+    <row r="33" ht="26" customHeight="1">
+      <c r="B33" s="46" t="inlineStr">
         <is>
           <t>KRITISCHER PFAD (ROT): V1 ➔ V2 ➔ V3 ➔ V4 ➔ V5 ➔ V6 ➔ V7 ➔ V8 ➔ V9 ➔ V11 ➔ V12 ➔ V13 ➔ V14  |  GESAMTDAUER: 46 ARBEITSTAGE</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="B35" s="46" t="inlineStr">
-        <is>
-          <t>Parallele Ausführung: V10 (Entsorgung Altdrucker) besitzt 1 Tag Gesamtpuffer (GP = 1, FP = 1) und beeinflusst das Projektende nicht, solange die Dauer ≤ 3 Tage bleibt.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="133">
+  <mergeCells count="127">
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="AD17:AE17"/>
     <mergeCell ref="N11:O11"/>
     <mergeCell ref="V17:W17"/>
-    <mergeCell ref="F29:G29"/>
     <mergeCell ref="Z11:AA11"/>
     <mergeCell ref="J19:K19"/>
     <mergeCell ref="R28:S28"/>
     <mergeCell ref="L19:M19"/>
-    <mergeCell ref="B31:C31"/>
     <mergeCell ref="J28:K28"/>
-    <mergeCell ref="D31:E31"/>
     <mergeCell ref="L28:M28"/>
     <mergeCell ref="L6:AM6"/>
     <mergeCell ref="V28:W28"/>
     <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B21:AM21"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="AF12:AG12"/>
@@ -2056,11 +2120,11 @@
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="F19:G19"/>
-    <mergeCell ref="B23:G23"/>
     <mergeCell ref="R12:W12"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="E6:G6"/>
     <mergeCell ref="H25:I25"/>
+    <mergeCell ref="F30:G30"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="V19:W19"/>
@@ -2068,26 +2132,25 @@
     <mergeCell ref="AD28:AE28"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="J11:K11"/>
-    <mergeCell ref="B29:C29"/>
     <mergeCell ref="T11:U11"/>
     <mergeCell ref="R18:W18"/>
     <mergeCell ref="V11:W11"/>
     <mergeCell ref="J18:O18"/>
-    <mergeCell ref="F31:G31"/>
     <mergeCell ref="N28:O28"/>
+    <mergeCell ref="F28:G28"/>
     <mergeCell ref="AH11:AI11"/>
     <mergeCell ref="N13:O13"/>
     <mergeCell ref="B25:G25"/>
     <mergeCell ref="B7:J7"/>
     <mergeCell ref="H12:I12"/>
     <mergeCell ref="Z27:AE27"/>
-    <mergeCell ref="D29:E29"/>
     <mergeCell ref="E8:G8"/>
     <mergeCell ref="H6:J6"/>
+    <mergeCell ref="B33:AM33"/>
     <mergeCell ref="J27:O27"/>
-    <mergeCell ref="B35:AM35"/>
     <mergeCell ref="Z12:AE12"/>
     <mergeCell ref="V13:W13"/>
+    <mergeCell ref="B29:G29"/>
     <mergeCell ref="Z26:AA26"/>
     <mergeCell ref="AB26:AC26"/>
     <mergeCell ref="B16:AM16"/>
@@ -2107,11 +2170,14 @@
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="AB11:AC11"/>
     <mergeCell ref="H8:J8"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="AD11:AE11"/>
+    <mergeCell ref="D28:E28"/>
     <mergeCell ref="N19:O19"/>
     <mergeCell ref="R17:S17"/>
     <mergeCell ref="T17:U17"/>
-    <mergeCell ref="B34:AM34"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
     <mergeCell ref="P12:Q12"/>
     <mergeCell ref="Z28:AA28"/>
     <mergeCell ref="T19:U19"/>
@@ -2120,10 +2186,9 @@
     <mergeCell ref="L11:M11"/>
     <mergeCell ref="T28:U28"/>
     <mergeCell ref="B18:G18"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="B15:AM15"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="X12:Y12"/>
+    <mergeCell ref="H29:I29"/>
     <mergeCell ref="R11:S11"/>
     <mergeCell ref="AJ11:AK11"/>
     <mergeCell ref="R27:W27"/>
@@ -2134,11 +2199,8 @@
     <mergeCell ref="L13:M13"/>
     <mergeCell ref="AD13:AE13"/>
     <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="J25:O25"/>
     <mergeCell ref="AJ13:AK13"/>
     <mergeCell ref="F26:G26"/>
-    <mergeCell ref="B30:G30"/>
     <mergeCell ref="AL13:AM13"/>
     <mergeCell ref="R26:S26"/>
     <mergeCell ref="L7:AM7"/>

</xml_diff>

<commit_message>
Design-Optimierung: Netzplan & PSP schlicht schwarz-weiss (nur kritischer Pfad rot), Legende ohne Text-Erklaerungen, Bereinigung alter/redundanter Daten
</commit_message>
<xml_diff>
--- a/docs/01_Projektorganisation/Netzplan.xlsx
+++ b/docs/01_Projektorganisation/Netzplan.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="34">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,34 +29,24 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <color rgb="00000000"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00595959"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="8.5"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="009C0006"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <sz val="8.5"/>
     </font>
     <font>
@@ -67,39 +57,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F497D"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002F5597"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F497D"/>
-      <sz val="10"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00000000"/>
-      <sz val="9"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -139,14 +103,8 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002F5597"/>
+      <color rgb="00000000"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002F5597"/>
-      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -157,26 +115,20 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002F5597"/>
+      <color rgb="00000000"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="009C0006"/>
-      <sz val="10.5"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10.5"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -196,29 +148,17 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002F5597"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F497D"/>
-      <sz val="11"/>
+      <color rgb="00000000"/>
+      <sz val="10.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="009C0006"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00404040"/>
-      <sz val="9.5"/>
+      <sz val="10.5"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -227,12 +167,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F497D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -242,32 +177,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00FFFDF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F5F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DEEBF7"/>
+        <fgColor rgb="00E6E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -432,7 +352,7 @@
         <color rgb="00D9D9D9"/>
       </right>
       <top style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
         <color rgb="00D9D9D9"/>
@@ -449,18 +369,18 @@
         <color rgb="00D9D9D9"/>
       </top>
       <bottom style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
     <border>
       <left style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
         <color rgb="00D9D9D9"/>
       </right>
       <top style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
         <color rgb="00D9D9D9"/>
@@ -471,10 +391,10 @@
         <color rgb="00D9D9D9"/>
       </left>
       <right style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </right>
       <top style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
         <color rgb="00D9D9D9"/>
@@ -482,7 +402,7 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
         <color rgb="00D9D9D9"/>
@@ -499,7 +419,7 @@
         <color rgb="00D9D9D9"/>
       </left>
       <right style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
         <color rgb="00D9D9D9"/>
@@ -510,7 +430,7 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
         <color rgb="00D9D9D9"/>
@@ -519,7 +439,7 @@
         <color rgb="00D9D9D9"/>
       </top>
       <bottom style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
     <border>
@@ -527,20 +447,20 @@
         <color rgb="00D9D9D9"/>
       </left>
       <right style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
         <color rgb="00D9D9D9"/>
       </top>
       <bottom style="medium">
-        <color rgb="002F5597"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -552,146 +472,129 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1107,14 +1010,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1"/>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Netzplan nach DIN 69900 (Knotenvorgangsmodell CPM)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
+    <row r="3" ht="18" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Projekt: IT-Ausstattung Planungs- und Konstruktionsbüro | Kunde: VektorPlan GmbH | Projektleiter: Jan Kluth | Gesamtdauer: 46 Arbeitstage</t>
@@ -1136,42 +1039,32 @@
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Pfade &amp; Farben:</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>FAZ (Früh. Start)</t>
         </is>
       </c>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="4" t="n"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Dauer (Tage)</t>
         </is>
       </c>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>FEZ (Früh. Ende)</t>
         </is>
       </c>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>■ KRITISCHER PFAD (Rot / Warmgelb): Gesamtpuffer GP = 0 (Verzögerung verschiebt Projektende).</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Vorgangs-Nr. &amp; Vorgangsbezeichnung (Kritisch = Roter Rahmen)</t>
         </is>
@@ -1184,644 +1077,634 @@
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4" t="n"/>
       <c r="J7" s="4" t="n"/>
-      <c r="L7" s="9" t="inlineStr">
-        <is>
-          <t>■ PARALLELER VORGANG MIT PUFFER (Blau): V10 (Entsorgung Altdrucker) läuft parallel zu V11 und hat GP = 1 Tag Puffer.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>SAZ (Spät. Start)</t>
         </is>
       </c>
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="4" t="n"/>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>GP (Gesamtpuffer)</t>
         </is>
       </c>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>SEZ (Spät. Ende)</t>
         </is>
       </c>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
-      <c r="L8" s="12" t="inlineStr">
-        <is>
-          <t>➔ Normalfolge (Ende-Anfang EA = 0): Nachfolger beginnt nach Ende des Vorgängers.</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  PHASE 1: PROJEKTSTART, SPEZIFIKATION &amp; PREISKALKULATION (TAGE 0 BIS 19)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1">
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>FAZ: 0</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>D: 2 T</t>
         </is>
       </c>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>FEZ: 2</t>
         </is>
       </c>
-      <c r="G11" s="17" t="n"/>
-      <c r="J11" s="14" t="inlineStr">
+      <c r="G11" s="12" t="n"/>
+      <c r="J11" s="9" t="inlineStr">
         <is>
           <t>FAZ: 2</t>
         </is>
       </c>
-      <c r="K11" s="15" t="n"/>
-      <c r="L11" s="16" t="inlineStr">
+      <c r="K11" s="10" t="n"/>
+      <c r="L11" s="11" t="inlineStr">
         <is>
           <t>D: 5 T</t>
         </is>
       </c>
-      <c r="M11" s="15" t="n"/>
-      <c r="N11" s="16" t="inlineStr">
+      <c r="M11" s="10" t="n"/>
+      <c r="N11" s="11" t="inlineStr">
         <is>
           <t>FEZ: 7</t>
         </is>
       </c>
-      <c r="O11" s="17" t="n"/>
-      <c r="R11" s="14" t="inlineStr">
+      <c r="O11" s="12" t="n"/>
+      <c r="R11" s="9" t="inlineStr">
         <is>
           <t>FAZ: 7</t>
         </is>
       </c>
-      <c r="S11" s="15" t="n"/>
-      <c r="T11" s="16" t="inlineStr">
+      <c r="S11" s="10" t="n"/>
+      <c r="T11" s="11" t="inlineStr">
         <is>
           <t>D: 5 T</t>
         </is>
       </c>
-      <c r="U11" s="15" t="n"/>
-      <c r="V11" s="16" t="inlineStr">
+      <c r="U11" s="10" t="n"/>
+      <c r="V11" s="11" t="inlineStr">
         <is>
           <t>FEZ: 12</t>
         </is>
       </c>
-      <c r="W11" s="17" t="n"/>
-      <c r="Z11" s="14" t="inlineStr">
+      <c r="W11" s="12" t="n"/>
+      <c r="Z11" s="9" t="inlineStr">
         <is>
           <t>FAZ: 12</t>
         </is>
       </c>
-      <c r="AA11" s="15" t="n"/>
-      <c r="AB11" s="16" t="inlineStr">
+      <c r="AA11" s="10" t="n"/>
+      <c r="AB11" s="11" t="inlineStr">
         <is>
           <t>D: 3 T</t>
         </is>
       </c>
-      <c r="AC11" s="15" t="n"/>
-      <c r="AD11" s="16" t="inlineStr">
+      <c r="AC11" s="10" t="n"/>
+      <c r="AD11" s="11" t="inlineStr">
         <is>
           <t>FEZ: 15</t>
         </is>
       </c>
-      <c r="AE11" s="17" t="n"/>
-      <c r="AH11" s="14" t="inlineStr">
+      <c r="AE11" s="12" t="n"/>
+      <c r="AH11" s="9" t="inlineStr">
         <is>
           <t>FAZ: 15</t>
         </is>
       </c>
-      <c r="AI11" s="15" t="n"/>
-      <c r="AJ11" s="16" t="inlineStr">
+      <c r="AI11" s="10" t="n"/>
+      <c r="AJ11" s="11" t="inlineStr">
         <is>
           <t>D: 4 T</t>
         </is>
       </c>
-      <c r="AK11" s="15" t="n"/>
-      <c r="AL11" s="16" t="inlineStr">
+      <c r="AK11" s="10" t="n"/>
+      <c r="AL11" s="11" t="inlineStr">
         <is>
           <t>FEZ: 19</t>
         </is>
       </c>
-      <c r="AM11" s="17" t="n"/>
+      <c r="AM11" s="12" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>V1: Projektstart &amp; Kick-off
 [Jan Kluth]</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="14" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="J12" s="18" t="inlineStr">
+      <c r="J12" s="13" t="inlineStr">
         <is>
           <t>V2: Anforderung &amp; Lastenheft
 [Mathias Vonau]</t>
         </is>
       </c>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" s="19" t="n"/>
-      <c r="M12" s="19" t="n"/>
-      <c r="N12" s="19" t="n"/>
-      <c r="O12" s="20" t="n"/>
-      <c r="P12" s="21" t="inlineStr">
+      <c r="K12" s="14" t="n"/>
+      <c r="L12" s="14" t="n"/>
+      <c r="M12" s="14" t="n"/>
+      <c r="N12" s="14" t="n"/>
+      <c r="O12" s="15" t="n"/>
+      <c r="P12" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="R12" s="18" t="inlineStr">
+      <c r="R12" s="13" t="inlineStr">
         <is>
           <t>V3: Marktrecherche Hardware
 [Marian Bolecke]</t>
         </is>
       </c>
-      <c r="S12" s="19" t="n"/>
-      <c r="T12" s="19" t="n"/>
-      <c r="U12" s="19" t="n"/>
-      <c r="V12" s="19" t="n"/>
-      <c r="W12" s="20" t="n"/>
-      <c r="X12" s="21" t="inlineStr">
+      <c r="S12" s="14" t="n"/>
+      <c r="T12" s="14" t="n"/>
+      <c r="U12" s="14" t="n"/>
+      <c r="V12" s="14" t="n"/>
+      <c r="W12" s="15" t="n"/>
+      <c r="X12" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="Z12" s="18" t="inlineStr">
+      <c r="Z12" s="13" t="inlineStr">
         <is>
           <t>V4: Nutzwertanalyse (NWA)
 [Marian Bolecke]</t>
         </is>
       </c>
-      <c r="AA12" s="19" t="n"/>
-      <c r="AB12" s="19" t="n"/>
-      <c r="AC12" s="19" t="n"/>
-      <c r="AD12" s="19" t="n"/>
-      <c r="AE12" s="20" t="n"/>
-      <c r="AF12" s="21" t="inlineStr">
+      <c r="AA12" s="14" t="n"/>
+      <c r="AB12" s="14" t="n"/>
+      <c r="AC12" s="14" t="n"/>
+      <c r="AD12" s="14" t="n"/>
+      <c r="AE12" s="15" t="n"/>
+      <c r="AF12" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="AH12" s="18" t="inlineStr">
+      <c r="AH12" s="13" t="inlineStr">
         <is>
           <t>V5: Angebot &amp; Kalkulation
 [Marian Bolecke]</t>
         </is>
       </c>
-      <c r="AI12" s="19" t="n"/>
-      <c r="AJ12" s="19" t="n"/>
-      <c r="AK12" s="19" t="n"/>
-      <c r="AL12" s="19" t="n"/>
-      <c r="AM12" s="20" t="n"/>
+      <c r="AI12" s="14" t="n"/>
+      <c r="AJ12" s="14" t="n"/>
+      <c r="AK12" s="14" t="n"/>
+      <c r="AL12" s="14" t="n"/>
+      <c r="AM12" s="15" t="n"/>
     </row>
     <row r="13" ht="19" customHeight="1">
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>SAZ: 0</t>
         </is>
       </c>
-      <c r="C13" s="23" t="n"/>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="E13" s="23" t="n"/>
-      <c r="F13" s="25" t="inlineStr">
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="20" t="inlineStr">
         <is>
           <t>SEZ: 2</t>
         </is>
       </c>
-      <c r="G13" s="26" t="n"/>
-      <c r="J13" s="22" t="inlineStr">
+      <c r="G13" s="21" t="n"/>
+      <c r="J13" s="17" t="inlineStr">
         <is>
           <t>SAZ: 2</t>
         </is>
       </c>
-      <c r="K13" s="23" t="n"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="K13" s="18" t="n"/>
+      <c r="L13" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="M13" s="23" t="n"/>
-      <c r="N13" s="25" t="inlineStr">
+      <c r="M13" s="18" t="n"/>
+      <c r="N13" s="20" t="inlineStr">
         <is>
           <t>SEZ: 7</t>
         </is>
       </c>
-      <c r="O13" s="26" t="n"/>
-      <c r="R13" s="22" t="inlineStr">
+      <c r="O13" s="21" t="n"/>
+      <c r="R13" s="17" t="inlineStr">
         <is>
           <t>SAZ: 7</t>
         </is>
       </c>
-      <c r="S13" s="23" t="n"/>
-      <c r="T13" s="24" t="inlineStr">
+      <c r="S13" s="18" t="n"/>
+      <c r="T13" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="U13" s="23" t="n"/>
-      <c r="V13" s="25" t="inlineStr">
+      <c r="U13" s="18" t="n"/>
+      <c r="V13" s="20" t="inlineStr">
         <is>
           <t>SEZ: 12</t>
         </is>
       </c>
-      <c r="W13" s="26" t="n"/>
-      <c r="Z13" s="22" t="inlineStr">
+      <c r="W13" s="21" t="n"/>
+      <c r="Z13" s="17" t="inlineStr">
         <is>
           <t>SAZ: 12</t>
         </is>
       </c>
-      <c r="AA13" s="23" t="n"/>
-      <c r="AB13" s="24" t="inlineStr">
+      <c r="AA13" s="18" t="n"/>
+      <c r="AB13" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="AC13" s="23" t="n"/>
-      <c r="AD13" s="25" t="inlineStr">
+      <c r="AC13" s="18" t="n"/>
+      <c r="AD13" s="20" t="inlineStr">
         <is>
           <t>SEZ: 15</t>
         </is>
       </c>
-      <c r="AE13" s="26" t="n"/>
-      <c r="AH13" s="22" t="inlineStr">
+      <c r="AE13" s="21" t="n"/>
+      <c r="AH13" s="17" t="inlineStr">
         <is>
           <t>SAZ: 15</t>
         </is>
       </c>
-      <c r="AI13" s="23" t="n"/>
-      <c r="AJ13" s="24" t="inlineStr">
+      <c r="AI13" s="18" t="n"/>
+      <c r="AJ13" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="AK13" s="23" t="n"/>
-      <c r="AL13" s="25" t="inlineStr">
+      <c r="AK13" s="18" t="n"/>
+      <c r="AL13" s="20" t="inlineStr">
         <is>
           <t>SEZ: 19</t>
         </is>
       </c>
-      <c r="AM13" s="26" t="n"/>
+      <c r="AM13" s="21" t="n"/>
     </row>
     <row r="14" ht="12" customHeight="1">
-      <c r="AK14" s="27" t="inlineStr">
+      <c r="AK14" s="22" t="inlineStr">
         <is>
           <t>│</t>
         </is>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
-      <c r="E15" s="28" t="inlineStr">
+      <c r="E15" s="23" t="inlineStr">
         <is>
           <t>▼</t>
         </is>
       </c>
-      <c r="F15" s="29" t="n"/>
-      <c r="G15" s="29" t="n"/>
-      <c r="H15" s="29" t="n"/>
-      <c r="I15" s="29" t="n"/>
-      <c r="J15" s="29" t="n"/>
-      <c r="K15" s="29" t="n"/>
-      <c r="L15" s="29" t="n"/>
-      <c r="M15" s="29" t="n"/>
-      <c r="N15" s="29" t="n"/>
-      <c r="O15" s="29" t="n"/>
-      <c r="P15" s="29" t="n"/>
-      <c r="Q15" s="29" t="n"/>
-      <c r="R15" s="29" t="n"/>
-      <c r="S15" s="29" t="n"/>
-      <c r="T15" s="29" t="n"/>
-      <c r="U15" s="29" t="n"/>
-      <c r="V15" s="29" t="n"/>
-      <c r="W15" s="29" t="n"/>
-      <c r="X15" s="29" t="n"/>
-      <c r="Y15" s="29" t="n"/>
-      <c r="Z15" s="29" t="n"/>
-      <c r="AA15" s="29" t="n"/>
-      <c r="AB15" s="29" t="n"/>
-      <c r="AC15" s="29" t="n"/>
-      <c r="AD15" s="29" t="n"/>
-      <c r="AE15" s="29" t="n"/>
-      <c r="AF15" s="29" t="n"/>
-      <c r="AG15" s="29" t="n"/>
-      <c r="AH15" s="29" t="n"/>
-      <c r="AI15" s="29" t="n"/>
-      <c r="AJ15" s="29" t="n"/>
-      <c r="AK15" s="29" t="n"/>
+      <c r="F15" s="24" t="n"/>
+      <c r="G15" s="24" t="n"/>
+      <c r="H15" s="24" t="n"/>
+      <c r="I15" s="24" t="n"/>
+      <c r="J15" s="24" t="n"/>
+      <c r="K15" s="24" t="n"/>
+      <c r="L15" s="24" t="n"/>
+      <c r="M15" s="24" t="n"/>
+      <c r="N15" s="24" t="n"/>
+      <c r="O15" s="24" t="n"/>
+      <c r="P15" s="24" t="n"/>
+      <c r="Q15" s="24" t="n"/>
+      <c r="R15" s="24" t="n"/>
+      <c r="S15" s="24" t="n"/>
+      <c r="T15" s="24" t="n"/>
+      <c r="U15" s="24" t="n"/>
+      <c r="V15" s="24" t="n"/>
+      <c r="W15" s="24" t="n"/>
+      <c r="X15" s="24" t="n"/>
+      <c r="Y15" s="24" t="n"/>
+      <c r="Z15" s="24" t="n"/>
+      <c r="AA15" s="24" t="n"/>
+      <c r="AB15" s="24" t="n"/>
+      <c r="AC15" s="24" t="n"/>
+      <c r="AD15" s="24" t="n"/>
+      <c r="AE15" s="24" t="n"/>
+      <c r="AF15" s="24" t="n"/>
+      <c r="AG15" s="24" t="n"/>
+      <c r="AH15" s="24" t="n"/>
+      <c r="AI15" s="24" t="n"/>
+      <c r="AJ15" s="24" t="n"/>
+      <c r="AK15" s="24" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  PHASE 2: BEAUFTRAGUNG, BESCHAFFUNG &amp; VORINSTALLATION / STAGING (TAGE 19 BIS 39)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1">
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>FAZ: 19</t>
         </is>
       </c>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>D: 3 T</t>
         </is>
       </c>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>FEZ: 22</t>
         </is>
       </c>
-      <c r="G17" s="17" t="n"/>
-      <c r="J17" s="14" t="inlineStr">
+      <c r="G17" s="12" t="n"/>
+      <c r="J17" s="9" t="inlineStr">
         <is>
           <t>FAZ: 22</t>
         </is>
       </c>
-      <c r="K17" s="15" t="n"/>
-      <c r="L17" s="16" t="inlineStr">
+      <c r="K17" s="10" t="n"/>
+      <c r="L17" s="11" t="inlineStr">
         <is>
           <t>D: 10 T</t>
         </is>
       </c>
-      <c r="M17" s="15" t="n"/>
-      <c r="N17" s="16" t="inlineStr">
+      <c r="M17" s="10" t="n"/>
+      <c r="N17" s="11" t="inlineStr">
         <is>
           <t>FEZ: 32</t>
         </is>
       </c>
-      <c r="O17" s="17" t="n"/>
-      <c r="R17" s="14" t="inlineStr">
+      <c r="O17" s="12" t="n"/>
+      <c r="R17" s="9" t="inlineStr">
         <is>
           <t>FAZ: 32</t>
         </is>
       </c>
-      <c r="S17" s="15" t="n"/>
-      <c r="T17" s="16" t="inlineStr">
+      <c r="S17" s="10" t="n"/>
+      <c r="T17" s="11" t="inlineStr">
         <is>
           <t>D: 2 T</t>
         </is>
       </c>
-      <c r="U17" s="15" t="n"/>
-      <c r="V17" s="16" t="inlineStr">
+      <c r="U17" s="10" t="n"/>
+      <c r="V17" s="11" t="inlineStr">
         <is>
           <t>FEZ: 34</t>
         </is>
       </c>
-      <c r="W17" s="17" t="n"/>
-      <c r="Z17" s="14" t="inlineStr">
+      <c r="W17" s="12" t="n"/>
+      <c r="Z17" s="9" t="inlineStr">
         <is>
           <t>FAZ: 34</t>
         </is>
       </c>
-      <c r="AA17" s="15" t="n"/>
-      <c r="AB17" s="16" t="inlineStr">
+      <c r="AA17" s="10" t="n"/>
+      <c r="AB17" s="11" t="inlineStr">
         <is>
           <t>D: 5 T</t>
         </is>
       </c>
-      <c r="AC17" s="15" t="n"/>
-      <c r="AD17" s="16" t="inlineStr">
+      <c r="AC17" s="10" t="n"/>
+      <c r="AD17" s="11" t="inlineStr">
         <is>
           <t>FEZ: 39</t>
         </is>
       </c>
-      <c r="AE17" s="17" t="n"/>
+      <c r="AE17" s="12" t="n"/>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>V6: Kundenfreigabe / Auftrag
 [Jan Kluth]</t>
         </is>
       </c>
-      <c r="C18" s="19" t="n"/>
-      <c r="D18" s="19" t="n"/>
-      <c r="E18" s="19" t="n"/>
-      <c r="F18" s="19" t="n"/>
-      <c r="G18" s="20" t="n"/>
-      <c r="H18" s="21" t="inlineStr">
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="14" t="n"/>
+      <c r="E18" s="14" t="n"/>
+      <c r="F18" s="14" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="J18" s="18" t="inlineStr">
+      <c r="J18" s="13" t="inlineStr">
         <is>
           <t>V7: Bestellung &amp; Beschaffung
 [Marian Bolecke]</t>
         </is>
       </c>
-      <c r="K18" s="19" t="n"/>
-      <c r="L18" s="19" t="n"/>
-      <c r="M18" s="19" t="n"/>
-      <c r="N18" s="19" t="n"/>
-      <c r="O18" s="20" t="n"/>
-      <c r="P18" s="21" t="inlineStr">
+      <c r="K18" s="14" t="n"/>
+      <c r="L18" s="14" t="n"/>
+      <c r="M18" s="14" t="n"/>
+      <c r="N18" s="14" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="R18" s="18" t="inlineStr">
+      <c r="R18" s="13" t="inlineStr">
         <is>
           <t>V8: Prüfung nach § 377 HGB
 [Marco Schmidt]</t>
         </is>
       </c>
-      <c r="S18" s="19" t="n"/>
-      <c r="T18" s="19" t="n"/>
-      <c r="U18" s="19" t="n"/>
-      <c r="V18" s="19" t="n"/>
-      <c r="W18" s="20" t="n"/>
-      <c r="X18" s="21" t="inlineStr">
+      <c r="S18" s="14" t="n"/>
+      <c r="T18" s="14" t="n"/>
+      <c r="U18" s="14" t="n"/>
+      <c r="V18" s="14" t="n"/>
+      <c r="W18" s="15" t="n"/>
+      <c r="X18" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="Z18" s="18" t="inlineStr">
+      <c r="Z18" s="13" t="inlineStr">
         <is>
           <t>V9: Vorinstallation &amp; Staging
 [Mathias &amp; Siyar]</t>
         </is>
       </c>
-      <c r="AA18" s="19" t="n"/>
-      <c r="AB18" s="19" t="n"/>
-      <c r="AC18" s="19" t="n"/>
-      <c r="AD18" s="19" t="n"/>
-      <c r="AE18" s="20" t="n"/>
+      <c r="AA18" s="14" t="n"/>
+      <c r="AB18" s="14" t="n"/>
+      <c r="AC18" s="14" t="n"/>
+      <c r="AD18" s="14" t="n"/>
+      <c r="AE18" s="15" t="n"/>
     </row>
     <row r="19" ht="19" customHeight="1">
-      <c r="B19" s="22" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>SAZ: 19</t>
         </is>
       </c>
-      <c r="C19" s="23" t="n"/>
-      <c r="D19" s="24" t="inlineStr">
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="25" t="inlineStr">
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="20" t="inlineStr">
         <is>
           <t>SEZ: 22</t>
         </is>
       </c>
-      <c r="G19" s="26" t="n"/>
-      <c r="J19" s="22" t="inlineStr">
+      <c r="G19" s="21" t="n"/>
+      <c r="J19" s="17" t="inlineStr">
         <is>
           <t>SAZ: 22</t>
         </is>
       </c>
-      <c r="K19" s="23" t="n"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="K19" s="18" t="n"/>
+      <c r="L19" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="M19" s="23" t="n"/>
-      <c r="N19" s="25" t="inlineStr">
+      <c r="M19" s="18" t="n"/>
+      <c r="N19" s="20" t="inlineStr">
         <is>
           <t>SEZ: 32</t>
         </is>
       </c>
-      <c r="O19" s="26" t="n"/>
-      <c r="R19" s="22" t="inlineStr">
+      <c r="O19" s="21" t="n"/>
+      <c r="R19" s="17" t="inlineStr">
         <is>
           <t>SAZ: 32</t>
         </is>
       </c>
-      <c r="S19" s="23" t="n"/>
-      <c r="T19" s="24" t="inlineStr">
+      <c r="S19" s="18" t="n"/>
+      <c r="T19" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="U19" s="23" t="n"/>
-      <c r="V19" s="25" t="inlineStr">
+      <c r="U19" s="18" t="n"/>
+      <c r="V19" s="20" t="inlineStr">
         <is>
           <t>SEZ: 34</t>
         </is>
       </c>
-      <c r="W19" s="26" t="n"/>
-      <c r="Z19" s="22" t="inlineStr">
+      <c r="W19" s="21" t="n"/>
+      <c r="Z19" s="17" t="inlineStr">
         <is>
           <t>SAZ: 34</t>
         </is>
       </c>
-      <c r="AA19" s="23" t="n"/>
-      <c r="AB19" s="24" t="inlineStr">
+      <c r="AA19" s="18" t="n"/>
+      <c r="AB19" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="AC19" s="23" t="n"/>
-      <c r="AD19" s="25" t="inlineStr">
+      <c r="AC19" s="18" t="n"/>
+      <c r="AD19" s="20" t="inlineStr">
         <is>
           <t>SEZ: 39</t>
         </is>
       </c>
-      <c r="AE19" s="26" t="n"/>
+      <c r="AE19" s="21" t="n"/>
     </row>
     <row r="20" ht="12" customHeight="1">
-      <c r="AC20" s="27" t="inlineStr">
+      <c r="AC20" s="22" t="inlineStr">
         <is>
           <t>│</t>
         </is>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1">
-      <c r="E21" s="28" t="inlineStr">
+      <c r="E21" s="23" t="inlineStr">
         <is>
           <t>▼</t>
         </is>
       </c>
-      <c r="F21" s="29" t="n"/>
-      <c r="G21" s="29" t="n"/>
-      <c r="H21" s="29" t="n"/>
-      <c r="I21" s="29" t="n"/>
-      <c r="J21" s="29" t="n"/>
-      <c r="K21" s="29" t="n"/>
-      <c r="L21" s="29" t="n"/>
-      <c r="M21" s="29" t="n"/>
-      <c r="N21" s="29" t="n"/>
-      <c r="O21" s="29" t="n"/>
-      <c r="P21" s="29" t="n"/>
-      <c r="Q21" s="29" t="n"/>
-      <c r="R21" s="29" t="n"/>
-      <c r="S21" s="29" t="n"/>
-      <c r="T21" s="29" t="n"/>
-      <c r="U21" s="29" t="n"/>
-      <c r="V21" s="29" t="n"/>
-      <c r="W21" s="29" t="n"/>
-      <c r="X21" s="29" t="n"/>
-      <c r="Y21" s="29" t="n"/>
-      <c r="Z21" s="29" t="n"/>
-      <c r="AA21" s="29" t="n"/>
-      <c r="AB21" s="29" t="n"/>
-      <c r="AC21" s="29" t="n"/>
+      <c r="F21" s="24" t="n"/>
+      <c r="G21" s="24" t="n"/>
+      <c r="H21" s="24" t="n"/>
+      <c r="I21" s="24" t="n"/>
+      <c r="J21" s="24" t="n"/>
+      <c r="K21" s="24" t="n"/>
+      <c r="L21" s="24" t="n"/>
+      <c r="M21" s="24" t="n"/>
+      <c r="N21" s="24" t="n"/>
+      <c r="O21" s="24" t="n"/>
+      <c r="P21" s="24" t="n"/>
+      <c r="Q21" s="24" t="n"/>
+      <c r="R21" s="24" t="n"/>
+      <c r="S21" s="24" t="n"/>
+      <c r="T21" s="24" t="n"/>
+      <c r="U21" s="24" t="n"/>
+      <c r="V21" s="24" t="n"/>
+      <c r="W21" s="24" t="n"/>
+      <c r="X21" s="24" t="n"/>
+      <c r="Y21" s="24" t="n"/>
+      <c r="Z21" s="24" t="n"/>
+      <c r="AA21" s="24" t="n"/>
+      <c r="AB21" s="24" t="n"/>
+      <c r="AC21" s="24" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PHASE 3: PARALLELE AUSFÜHRUNG (V10 || V11), ROLLOUT &amp; ABSCHLUSS (TAGE 39 BIS 46)</t>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PHASE 3: PARALLELE AUSFÜHRUNG, ROLLOUT &amp; ABSCHLUSS (TAGE 39 BIS 46)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="14" customHeight="1">
-      <c r="E23" s="30" t="inlineStr">
+      <c r="E23" s="25" t="inlineStr">
         <is>
           <t>▼</t>
         </is>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="B24" s="31" t="inlineStr">
+      <c r="B24" s="26" t="inlineStr">
         <is>
           <t>FAZ: 39</t>
         </is>
       </c>
-      <c r="C24" s="32" t="n"/>
-      <c r="D24" s="33" t="inlineStr">
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="28" t="inlineStr">
         <is>
           <t>D: 2 T</t>
         </is>
       </c>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="33" t="inlineStr">
+      <c r="E24" s="27" t="n"/>
+      <c r="F24" s="28" t="inlineStr">
         <is>
           <t>FEZ: 41</t>
         </is>
       </c>
-      <c r="G24" s="34" t="n"/>
+      <c r="G24" s="29" t="n"/>
     </row>
     <row r="25" ht="32" customHeight="1">
-      <c r="B25" s="35" t="inlineStr">
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t>V10: Entsorgung Altdrucker
 [Marco Schmidt]</t>
@@ -1831,264 +1714,264 @@
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="36" t="n"/>
-      <c r="H25" s="37" t="inlineStr">
+      <c r="G25" s="31" t="n"/>
+      <c r="H25" s="32" t="inlineStr">
         <is>
           <t>➔ ↘</t>
         </is>
       </c>
     </row>
     <row r="26" ht="19" customHeight="1">
-      <c r="B26" s="38" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
         <is>
           <t>SAZ: 40</t>
         </is>
       </c>
-      <c r="C26" s="39" t="n"/>
-      <c r="D26" s="40" t="inlineStr">
+      <c r="C26" s="34" t="n"/>
+      <c r="D26" s="35" t="inlineStr">
         <is>
           <t>GP: 1 T</t>
         </is>
       </c>
-      <c r="E26" s="39" t="n"/>
-      <c r="F26" s="41" t="inlineStr">
+      <c r="E26" s="34" t="n"/>
+      <c r="F26" s="36" t="inlineStr">
         <is>
           <t>SEZ: 42</t>
         </is>
       </c>
-      <c r="G26" s="42" t="n"/>
-      <c r="J26" s="14" t="inlineStr">
+      <c r="G26" s="37" t="n"/>
+      <c r="J26" s="9" t="inlineStr">
         <is>
           <t>FAZ: 42</t>
         </is>
       </c>
-      <c r="K26" s="15" t="n"/>
-      <c r="L26" s="16" t="inlineStr">
+      <c r="K26" s="10" t="n"/>
+      <c r="L26" s="11" t="inlineStr">
         <is>
           <t>D: 2 T</t>
         </is>
       </c>
-      <c r="M26" s="15" t="n"/>
-      <c r="N26" s="16" t="inlineStr">
+      <c r="M26" s="10" t="n"/>
+      <c r="N26" s="11" t="inlineStr">
         <is>
           <t>FEZ: 44</t>
         </is>
       </c>
-      <c r="O26" s="17" t="n"/>
-      <c r="R26" s="14" t="inlineStr">
+      <c r="O26" s="12" t="n"/>
+      <c r="R26" s="9" t="inlineStr">
         <is>
           <t>FAZ: 44</t>
         </is>
       </c>
-      <c r="S26" s="15" t="n"/>
-      <c r="T26" s="16" t="inlineStr">
+      <c r="S26" s="10" t="n"/>
+      <c r="T26" s="11" t="inlineStr">
         <is>
           <t>D: 1 T</t>
         </is>
       </c>
-      <c r="U26" s="15" t="n"/>
-      <c r="V26" s="16" t="inlineStr">
+      <c r="U26" s="10" t="n"/>
+      <c r="V26" s="11" t="inlineStr">
         <is>
           <t>FEZ: 45</t>
         </is>
       </c>
-      <c r="W26" s="17" t="n"/>
-      <c r="Z26" s="14" t="inlineStr">
+      <c r="W26" s="12" t="n"/>
+      <c r="Z26" s="9" t="inlineStr">
         <is>
           <t>FAZ: 45</t>
         </is>
       </c>
-      <c r="AA26" s="15" t="n"/>
-      <c r="AB26" s="16" t="inlineStr">
+      <c r="AA26" s="10" t="n"/>
+      <c r="AB26" s="11" t="inlineStr">
         <is>
           <t>D: 1 T</t>
         </is>
       </c>
-      <c r="AC26" s="15" t="n"/>
-      <c r="AD26" s="16" t="inlineStr">
+      <c r="AC26" s="10" t="n"/>
+      <c r="AD26" s="11" t="inlineStr">
         <is>
           <t>FEZ: 46</t>
         </is>
       </c>
-      <c r="AE26" s="17" t="n"/>
+      <c r="AE26" s="12" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="E27" s="43" t="inlineStr">
+      <c r="E27" s="38" t="inlineStr">
         <is>
           <t>│  ▼</t>
         </is>
       </c>
-      <c r="I27" s="44" t="inlineStr">
+      <c r="I27" s="39" t="inlineStr">
         <is>
           <t>►</t>
         </is>
       </c>
-      <c r="J27" s="18" t="inlineStr">
+      <c r="J27" s="13" t="inlineStr">
         <is>
           <t>V12: Funktionstest &amp; Abnahme
 [Gesamtes Team]</t>
         </is>
       </c>
-      <c r="K27" s="19" t="n"/>
-      <c r="L27" s="19" t="n"/>
-      <c r="M27" s="19" t="n"/>
-      <c r="N27" s="19" t="n"/>
-      <c r="O27" s="20" t="n"/>
-      <c r="P27" s="21" t="inlineStr">
+      <c r="K27" s="14" t="n"/>
+      <c r="L27" s="14" t="n"/>
+      <c r="M27" s="14" t="n"/>
+      <c r="N27" s="14" t="n"/>
+      <c r="O27" s="15" t="n"/>
+      <c r="P27" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="R27" s="18" t="inlineStr">
+      <c r="R27" s="13" t="inlineStr">
         <is>
           <t>V13: Übergabe &amp; Dokumentation
 [Jan Kluth]</t>
         </is>
       </c>
-      <c r="S27" s="19" t="n"/>
-      <c r="T27" s="19" t="n"/>
-      <c r="U27" s="19" t="n"/>
-      <c r="V27" s="19" t="n"/>
-      <c r="W27" s="20" t="n"/>
-      <c r="X27" s="21" t="inlineStr">
+      <c r="S27" s="14" t="n"/>
+      <c r="T27" s="14" t="n"/>
+      <c r="U27" s="14" t="n"/>
+      <c r="V27" s="14" t="n"/>
+      <c r="W27" s="15" t="n"/>
+      <c r="X27" s="16" t="inlineStr">
         <is>
           <t>➔</t>
         </is>
       </c>
-      <c r="Z27" s="18" t="inlineStr">
+      <c r="Z27" s="13" t="inlineStr">
         <is>
           <t>V14: Lessons Learned &amp; Abschluss
 [Gesamtes Team]</t>
         </is>
       </c>
-      <c r="AA27" s="19" t="n"/>
-      <c r="AB27" s="19" t="n"/>
-      <c r="AC27" s="19" t="n"/>
-      <c r="AD27" s="19" t="n"/>
-      <c r="AE27" s="20" t="n"/>
+      <c r="AA27" s="14" t="n"/>
+      <c r="AB27" s="14" t="n"/>
+      <c r="AC27" s="14" t="n"/>
+      <c r="AD27" s="14" t="n"/>
+      <c r="AE27" s="15" t="n"/>
     </row>
     <row r="28" ht="19" customHeight="1">
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>FAZ: 39</t>
         </is>
       </c>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>D: 3 T</t>
         </is>
       </c>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>FEZ: 42</t>
         </is>
       </c>
-      <c r="G28" s="17" t="n"/>
-      <c r="J28" s="22" t="inlineStr">
+      <c r="G28" s="12" t="n"/>
+      <c r="J28" s="17" t="inlineStr">
         <is>
           <t>SAZ: 42</t>
         </is>
       </c>
-      <c r="K28" s="23" t="n"/>
-      <c r="L28" s="24" t="inlineStr">
+      <c r="K28" s="18" t="n"/>
+      <c r="L28" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="M28" s="23" t="n"/>
-      <c r="N28" s="25" t="inlineStr">
+      <c r="M28" s="18" t="n"/>
+      <c r="N28" s="20" t="inlineStr">
         <is>
           <t>SEZ: 44</t>
         </is>
       </c>
-      <c r="O28" s="26" t="n"/>
-      <c r="R28" s="22" t="inlineStr">
+      <c r="O28" s="21" t="n"/>
+      <c r="R28" s="17" t="inlineStr">
         <is>
           <t>SAZ: 44</t>
         </is>
       </c>
-      <c r="S28" s="23" t="n"/>
-      <c r="T28" s="24" t="inlineStr">
+      <c r="S28" s="18" t="n"/>
+      <c r="T28" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="U28" s="23" t="n"/>
-      <c r="V28" s="25" t="inlineStr">
+      <c r="U28" s="18" t="n"/>
+      <c r="V28" s="20" t="inlineStr">
         <is>
           <t>SEZ: 45</t>
         </is>
       </c>
-      <c r="W28" s="26" t="n"/>
-      <c r="Z28" s="22" t="inlineStr">
+      <c r="W28" s="21" t="n"/>
+      <c r="Z28" s="17" t="inlineStr">
         <is>
           <t>SAZ: 45</t>
         </is>
       </c>
-      <c r="AA28" s="23" t="n"/>
-      <c r="AB28" s="24" t="inlineStr">
+      <c r="AA28" s="18" t="n"/>
+      <c r="AB28" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="AC28" s="23" t="n"/>
-      <c r="AD28" s="25" t="inlineStr">
+      <c r="AC28" s="18" t="n"/>
+      <c r="AD28" s="20" t="inlineStr">
         <is>
           <t>SEZ: 46</t>
         </is>
       </c>
-      <c r="AE28" s="26" t="n"/>
+      <c r="AE28" s="21" t="n"/>
     </row>
     <row r="29" ht="32" customHeight="1">
-      <c r="B29" s="18" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>V11: Lieferung &amp; Montage vor Ort
 [Mathias &amp; Siyar]</t>
         </is>
       </c>
-      <c r="C29" s="19" t="n"/>
-      <c r="D29" s="19" t="n"/>
-      <c r="E29" s="19" t="n"/>
-      <c r="F29" s="19" t="n"/>
-      <c r="G29" s="20" t="n"/>
-      <c r="H29" s="45" t="inlineStr">
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="40" t="inlineStr">
         <is>
           <t>➔ ↗</t>
         </is>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1">
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>SAZ: 39</t>
         </is>
       </c>
-      <c r="C30" s="23" t="n"/>
-      <c r="D30" s="24" t="inlineStr">
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>GP: 0</t>
         </is>
       </c>
-      <c r="E30" s="23" t="n"/>
-      <c r="F30" s="25" t="inlineStr">
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="20" t="inlineStr">
         <is>
           <t>SEZ: 42</t>
         </is>
       </c>
-      <c r="G30" s="26" t="n"/>
+      <c r="G30" s="21" t="n"/>
     </row>
     <row r="32" ht="10" customHeight="1"/>
-    <row r="33" ht="26" customHeight="1">
-      <c r="B33" s="46" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="B33" s="41" t="inlineStr">
         <is>
           <t>KRITISCHER PFAD (ROT): V1 ➔ V2 ➔ V3 ➔ V4 ➔ V5 ➔ V6 ➔ V7 ➔ V8 ➔ V9 ➔ V11 ➔ V12 ➔ V13 ➔ V14  |  GESAMTDAUER: 46 ARBEITSTAGE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="127">
+  <mergeCells count="123">
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="AD17:AE17"/>
     <mergeCell ref="N11:O11"/>
@@ -2099,7 +1982,6 @@
     <mergeCell ref="L19:M19"/>
     <mergeCell ref="J28:K28"/>
     <mergeCell ref="L28:M28"/>
-    <mergeCell ref="L6:AM6"/>
     <mergeCell ref="V28:W28"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="B6:D6"/>
@@ -2112,7 +1994,6 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="D24:E24"/>
     <mergeCell ref="B12:G12"/>
-    <mergeCell ref="L8:AM8"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="AH13:AI13"/>
     <mergeCell ref="D26:E26"/>
@@ -2182,7 +2063,6 @@
     <mergeCell ref="Z28:AA28"/>
     <mergeCell ref="T19:U19"/>
     <mergeCell ref="AB28:AC28"/>
-    <mergeCell ref="L5:AM5"/>
     <mergeCell ref="L11:M11"/>
     <mergeCell ref="T28:U28"/>
     <mergeCell ref="B18:G18"/>
@@ -2203,7 +2083,6 @@
     <mergeCell ref="F26:G26"/>
     <mergeCell ref="AL13:AM13"/>
     <mergeCell ref="R26:S26"/>
-    <mergeCell ref="L7:AM7"/>
     <mergeCell ref="T26:U26"/>
     <mergeCell ref="V26:W26"/>
     <mergeCell ref="T13:U13"/>
@@ -2227,7 +2106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2243,764 +2122,717 @@
     <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="47" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="42" t="inlineStr">
         <is>
           <t>Vorgangsknoten-Berechnungstabelle nach DIN 69900 (Knotenvorgangsmodell CPM)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="48" t="inlineStr">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="43" t="inlineStr">
         <is>
           <t>Vorgangs-Nr.</t>
         </is>
       </c>
-      <c r="B3" s="48" t="inlineStr">
+      <c r="B3" s="43" t="inlineStr">
         <is>
           <t>Vorgangsbezeichnung</t>
         </is>
       </c>
-      <c r="C3" s="48" t="inlineStr">
+      <c r="C3" s="43" t="inlineStr">
         <is>
           <t>Dauer (Tage)</t>
         </is>
       </c>
-      <c r="D3" s="48" t="inlineStr">
+      <c r="D3" s="43" t="inlineStr">
         <is>
           <t>Vorgänger</t>
         </is>
       </c>
-      <c r="E3" s="48" t="inlineStr">
+      <c r="E3" s="43" t="inlineStr">
         <is>
           <t>Nachfolger</t>
         </is>
       </c>
-      <c r="F3" s="48" t="inlineStr">
+      <c r="F3" s="43" t="inlineStr">
         <is>
           <t>FAZ (Frühester Anfang)</t>
         </is>
       </c>
-      <c r="G3" s="48" t="inlineStr">
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t>FEZ (Frühestes Ende)</t>
         </is>
       </c>
-      <c r="H3" s="48" t="inlineStr">
+      <c r="H3" s="43" t="inlineStr">
         <is>
           <t>SAZ (Spätester Anfang)</t>
         </is>
       </c>
-      <c r="I3" s="48" t="inlineStr">
+      <c r="I3" s="43" t="inlineStr">
         <is>
           <t>SEZ (Spätestes Ende)</t>
         </is>
       </c>
-      <c r="J3" s="48" t="inlineStr">
+      <c r="J3" s="43" t="inlineStr">
         <is>
           <t>Gesamtpuffer (GP)</t>
         </is>
       </c>
-      <c r="K3" s="48" t="inlineStr">
+      <c r="K3" s="43" t="inlineStr">
         <is>
           <t>Kritisch / Status</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="49" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="B4" s="50" t="inlineStr">
+      <c r="B4" s="45" t="inlineStr">
         <is>
           <t>Projektstart &amp; Kick-off-Meeting</t>
         </is>
       </c>
-      <c r="C4" s="49" t="n">
+      <c r="C4" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="51" t="inlineStr">
+      <c r="D4" s="46" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E4" s="51" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="F4" s="51" t="n">
+      <c r="F4" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="51" t="n">
+      <c r="G4" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="51" t="n">
+      <c r="H4" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="51" t="n">
+      <c r="I4" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="J4" s="52" t="n">
+      <c r="J4" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="49" t="inlineStr">
+      <c r="K4" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="49" t="inlineStr">
+      <c r="A5" s="44" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="B5" s="50" t="inlineStr">
+      <c r="B5" s="45" t="inlineStr">
         <is>
           <t>Anforderungsanalyse &amp; Lastenhefterstellung</t>
         </is>
       </c>
-      <c r="C5" s="49" t="n">
+      <c r="C5" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="51" t="inlineStr">
+      <c r="D5" s="46" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="E5" s="51" t="inlineStr">
+      <c r="E5" s="46" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
-      <c r="F5" s="51" t="n">
+      <c r="F5" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="51" t="n">
+      <c r="G5" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="H5" s="51" t="n">
+      <c r="H5" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="I5" s="51" t="n">
+      <c r="I5" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="J5" s="52" t="n">
+      <c r="J5" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="49" t="inlineStr">
+      <c r="K5" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="49" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
-      <c r="B6" s="50" t="inlineStr">
+      <c r="B6" s="45" t="inlineStr">
         <is>
           <t>Marktrecherche &amp; Einholen von Angeboten</t>
         </is>
       </c>
-      <c r="C6" s="49" t="n">
+      <c r="C6" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="51" t="inlineStr">
+      <c r="D6" s="46" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="E6" s="51" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
-      <c r="F6" s="51" t="n">
+      <c r="F6" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="G6" s="51" t="n">
+      <c r="G6" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="H6" s="51" t="n">
+      <c r="H6" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="I6" s="51" t="n">
+      <c r="I6" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="J6" s="52" t="n">
+      <c r="J6" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="49" t="inlineStr">
+      <c r="K6" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="49" t="inlineStr">
+      <c r="A7" s="44" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
-      <c r="B7" s="50" t="inlineStr">
+      <c r="B7" s="45" t="inlineStr">
         <is>
           <t>Nutzwertanalyse (Hardware-Auswahl)</t>
         </is>
       </c>
-      <c r="C7" s="49" t="n">
+      <c r="C7" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="51" t="inlineStr">
+      <c r="D7" s="46" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
-      <c r="E7" s="51" t="inlineStr">
+      <c r="E7" s="46" t="inlineStr">
         <is>
           <t>V5</t>
         </is>
       </c>
-      <c r="F7" s="51" t="n">
+      <c r="F7" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="G7" s="51" t="n">
+      <c r="G7" s="46" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="51" t="n">
+      <c r="H7" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="I7" s="51" t="n">
+      <c r="I7" s="46" t="n">
         <v>15</v>
       </c>
-      <c r="J7" s="52" t="n">
+      <c r="J7" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="49" t="inlineStr">
+      <c r="K7" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="49" t="inlineStr">
+      <c r="A8" s="44" t="inlineStr">
         <is>
           <t>V5</t>
         </is>
       </c>
-      <c r="B8" s="50" t="inlineStr">
+      <c r="B8" s="45" t="inlineStr">
         <is>
           <t>Angebotserstellung &amp; Vorwärtskalkulation</t>
         </is>
       </c>
-      <c r="C8" s="49" t="n">
+      <c r="C8" s="44" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="51" t="inlineStr">
+      <c r="D8" s="46" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
-      <c r="E8" s="51" t="inlineStr">
+      <c r="E8" s="46" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="F8" s="51" t="n">
+      <c r="F8" s="46" t="n">
         <v>15</v>
       </c>
-      <c r="G8" s="51" t="n">
+      <c r="G8" s="46" t="n">
         <v>19</v>
       </c>
-      <c r="H8" s="51" t="n">
+      <c r="H8" s="46" t="n">
         <v>15</v>
       </c>
-      <c r="I8" s="51" t="n">
+      <c r="I8" s="46" t="n">
         <v>19</v>
       </c>
-      <c r="J8" s="52" t="n">
+      <c r="J8" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="49" t="inlineStr">
+      <c r="K8" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="49" t="inlineStr">
+      <c r="A9" s="44" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="B9" s="50" t="inlineStr">
+      <c r="B9" s="45" t="inlineStr">
         <is>
           <t>Kundenfreigabe &amp; Auftragsvergabe</t>
         </is>
       </c>
-      <c r="C9" s="49" t="n">
+      <c r="C9" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="51" t="inlineStr">
+      <c r="D9" s="46" t="inlineStr">
         <is>
           <t>V5</t>
         </is>
       </c>
-      <c r="E9" s="51" t="inlineStr">
+      <c r="E9" s="46" t="inlineStr">
         <is>
           <t>V7</t>
         </is>
       </c>
-      <c r="F9" s="51" t="n">
+      <c r="F9" s="46" t="n">
         <v>19</v>
       </c>
-      <c r="G9" s="51" t="n">
+      <c r="G9" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="H9" s="51" t="n">
+      <c r="H9" s="46" t="n">
         <v>19</v>
       </c>
-      <c r="I9" s="51" t="n">
+      <c r="I9" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="J9" s="52" t="n">
+      <c r="J9" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="49" t="inlineStr">
+      <c r="K9" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="49" t="inlineStr">
+      <c r="A10" s="44" t="inlineStr">
         <is>
           <t>V7</t>
         </is>
       </c>
-      <c r="B10" s="50" t="inlineStr">
+      <c r="B10" s="45" t="inlineStr">
         <is>
           <t>Bestellung &amp; Beschaffung der Komponenten</t>
         </is>
       </c>
-      <c r="C10" s="49" t="n">
+      <c r="C10" s="44" t="n">
         <v>10</v>
       </c>
-      <c r="D10" s="51" t="inlineStr">
+      <c r="D10" s="46" t="inlineStr">
         <is>
           <t>V6</t>
         </is>
       </c>
-      <c r="E10" s="51" t="inlineStr">
+      <c r="E10" s="46" t="inlineStr">
         <is>
           <t>V8</t>
         </is>
       </c>
-      <c r="F10" s="51" t="n">
+      <c r="F10" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="G10" s="51" t="n">
+      <c r="G10" s="46" t="n">
         <v>32</v>
       </c>
-      <c r="H10" s="51" t="n">
+      <c r="H10" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="I10" s="51" t="n">
+      <c r="I10" s="46" t="n">
         <v>32</v>
       </c>
-      <c r="J10" s="52" t="n">
+      <c r="J10" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="49" t="inlineStr">
+      <c r="K10" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="49" t="inlineStr">
+      <c r="A11" s="44" t="inlineStr">
         <is>
           <t>V8</t>
         </is>
       </c>
-      <c r="B11" s="50" t="inlineStr">
+      <c r="B11" s="45" t="inlineStr">
         <is>
           <t>Wareneingangsprüfung nach § 377 HGB</t>
         </is>
       </c>
-      <c r="C11" s="49" t="n">
+      <c r="C11" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="51" t="inlineStr">
+      <c r="D11" s="46" t="inlineStr">
         <is>
           <t>V7</t>
         </is>
       </c>
-      <c r="E11" s="51" t="inlineStr">
+      <c r="E11" s="46" t="inlineStr">
         <is>
           <t>V9</t>
         </is>
       </c>
-      <c r="F11" s="51" t="n">
+      <c r="F11" s="46" t="n">
         <v>32</v>
       </c>
-      <c r="G11" s="51" t="n">
+      <c r="G11" s="46" t="n">
         <v>34</v>
       </c>
-      <c r="H11" s="51" t="n">
+      <c r="H11" s="46" t="n">
         <v>32</v>
       </c>
-      <c r="I11" s="51" t="n">
+      <c r="I11" s="46" t="n">
         <v>34</v>
       </c>
-      <c r="J11" s="52" t="n">
+      <c r="J11" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="49" t="inlineStr">
+      <c r="K11" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="49" t="inlineStr">
+      <c r="A12" s="44" t="inlineStr">
         <is>
           <t>V9</t>
         </is>
       </c>
-      <c r="B12" s="50" t="inlineStr">
+      <c r="B12" s="45" t="inlineStr">
         <is>
           <t>Vorinstallation, Konfiguration &amp; Staging</t>
         </is>
       </c>
-      <c r="C12" s="49" t="n">
+      <c r="C12" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="51" t="inlineStr">
+      <c r="D12" s="46" t="inlineStr">
         <is>
           <t>V8</t>
         </is>
       </c>
-      <c r="E12" s="51" t="inlineStr">
+      <c r="E12" s="46" t="inlineStr">
         <is>
           <t>V10, V11</t>
         </is>
       </c>
-      <c r="F12" s="51" t="n">
+      <c r="F12" s="46" t="n">
         <v>34</v>
       </c>
-      <c r="G12" s="51" t="n">
+      <c r="G12" s="46" t="n">
         <v>39</v>
       </c>
-      <c r="H12" s="51" t="n">
+      <c r="H12" s="46" t="n">
         <v>34</v>
       </c>
-      <c r="I12" s="51" t="n">
+      <c r="I12" s="46" t="n">
         <v>39</v>
       </c>
-      <c r="J12" s="52" t="n">
+      <c r="J12" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="49" t="inlineStr">
+      <c r="K12" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="53" t="inlineStr">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>V10</t>
         </is>
       </c>
-      <c r="B13" s="54" t="inlineStr">
+      <c r="B13" s="49" t="inlineStr">
         <is>
           <t>Fachgerechte Entsorgung Altdrucker (ElektroG)</t>
         </is>
       </c>
-      <c r="C13" s="53" t="n">
+      <c r="C13" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="55" t="inlineStr">
+      <c r="D13" s="50" t="inlineStr">
         <is>
           <t>V9</t>
         </is>
       </c>
-      <c r="E13" s="55" t="inlineStr">
+      <c r="E13" s="50" t="inlineStr">
         <is>
           <t>V12</t>
         </is>
       </c>
-      <c r="F13" s="55" t="n">
+      <c r="F13" s="50" t="n">
         <v>39</v>
       </c>
-      <c r="G13" s="55" t="n">
+      <c r="G13" s="50" t="n">
         <v>41</v>
       </c>
-      <c r="H13" s="55" t="n">
+      <c r="H13" s="50" t="n">
         <v>40</v>
       </c>
-      <c r="I13" s="55" t="n">
+      <c r="I13" s="50" t="n">
         <v>42</v>
       </c>
-      <c r="J13" s="56" t="n">
+      <c r="J13" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="K13" s="53" t="inlineStr">
+      <c r="K13" s="48" t="inlineStr">
         <is>
           <t>NEIN (1 Tag Puffer, parallel zu V11)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="49" t="inlineStr">
+      <c r="A14" s="44" t="inlineStr">
         <is>
           <t>V11</t>
         </is>
       </c>
-      <c r="B14" s="50" t="inlineStr">
+      <c r="B14" s="45" t="inlineStr">
         <is>
           <t>Lieferung, Montage &amp; Verkabelung vor Ort</t>
         </is>
       </c>
-      <c r="C14" s="49" t="n">
+      <c r="C14" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="51" t="inlineStr">
+      <c r="D14" s="46" t="inlineStr">
         <is>
           <t>V9</t>
         </is>
       </c>
-      <c r="E14" s="51" t="inlineStr">
+      <c r="E14" s="46" t="inlineStr">
         <is>
           <t>V12</t>
         </is>
       </c>
-      <c r="F14" s="51" t="n">
+      <c r="F14" s="46" t="n">
         <v>39</v>
       </c>
-      <c r="G14" s="51" t="n">
+      <c r="G14" s="46" t="n">
         <v>42</v>
       </c>
-      <c r="H14" s="51" t="n">
+      <c r="H14" s="46" t="n">
         <v>39</v>
       </c>
-      <c r="I14" s="51" t="n">
+      <c r="I14" s="46" t="n">
         <v>42</v>
       </c>
-      <c r="J14" s="52" t="n">
+      <c r="J14" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="49" t="inlineStr">
+      <c r="K14" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad, parallel zu V10)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="49" t="inlineStr">
+      <c r="A15" s="44" t="inlineStr">
         <is>
           <t>V12</t>
         </is>
       </c>
-      <c r="B15" s="50" t="inlineStr">
+      <c r="B15" s="45" t="inlineStr">
         <is>
           <t>Funktionstest &amp; Gesamtabnahme</t>
         </is>
       </c>
-      <c r="C15" s="49" t="n">
+      <c r="C15" s="44" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="51" t="inlineStr">
+      <c r="D15" s="46" t="inlineStr">
         <is>
           <t>V10, V11</t>
         </is>
       </c>
-      <c r="E15" s="51" t="inlineStr">
+      <c r="E15" s="46" t="inlineStr">
         <is>
           <t>V13</t>
         </is>
       </c>
-      <c r="F15" s="51" t="n">
+      <c r="F15" s="46" t="n">
         <v>42</v>
       </c>
-      <c r="G15" s="51" t="n">
+      <c r="G15" s="46" t="n">
         <v>44</v>
       </c>
-      <c r="H15" s="51" t="n">
+      <c r="H15" s="46" t="n">
         <v>42</v>
       </c>
-      <c r="I15" s="51" t="n">
+      <c r="I15" s="46" t="n">
         <v>44</v>
       </c>
-      <c r="J15" s="52" t="n">
+      <c r="J15" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="49" t="inlineStr">
+      <c r="K15" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="49" t="inlineStr">
+      <c r="A16" s="44" t="inlineStr">
         <is>
           <t>V13</t>
         </is>
       </c>
-      <c r="B16" s="50" t="inlineStr">
+      <c r="B16" s="45" t="inlineStr">
         <is>
           <t>Mitarbeitereinweisung &amp; formelle Übergabe</t>
         </is>
       </c>
-      <c r="C16" s="49" t="n">
+      <c r="C16" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="51" t="inlineStr">
+      <c r="D16" s="46" t="inlineStr">
         <is>
           <t>V12</t>
         </is>
       </c>
-      <c r="E16" s="51" t="inlineStr">
+      <c r="E16" s="46" t="inlineStr">
         <is>
           <t>V14</t>
         </is>
       </c>
-      <c r="F16" s="51" t="n">
+      <c r="F16" s="46" t="n">
         <v>44</v>
       </c>
-      <c r="G16" s="51" t="n">
+      <c r="G16" s="46" t="n">
         <v>45</v>
       </c>
-      <c r="H16" s="51" t="n">
+      <c r="H16" s="46" t="n">
         <v>44</v>
       </c>
-      <c r="I16" s="51" t="n">
+      <c r="I16" s="46" t="n">
         <v>45</v>
       </c>
-      <c r="J16" s="52" t="n">
+      <c r="J16" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="49" t="inlineStr">
+      <c r="K16" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="49" t="inlineStr">
+      <c r="A17" s="44" t="inlineStr">
         <is>
           <t>V14</t>
         </is>
       </c>
-      <c r="B17" s="50" t="inlineStr">
+      <c r="B17" s="45" t="inlineStr">
         <is>
           <t>Projektabschlussbericht &amp; Lessons Learned</t>
         </is>
       </c>
-      <c r="C17" s="49" t="n">
+      <c r="C17" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="51" t="inlineStr">
+      <c r="D17" s="46" t="inlineStr">
         <is>
           <t>V13</t>
         </is>
       </c>
-      <c r="E17" s="51" t="inlineStr">
+      <c r="E17" s="46" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="51" t="n">
+      <c r="F17" s="46" t="n">
         <v>45</v>
       </c>
-      <c r="G17" s="51" t="n">
+      <c r="G17" s="46" t="n">
         <v>46</v>
       </c>
-      <c r="H17" s="51" t="n">
+      <c r="H17" s="46" t="n">
         <v>45</v>
       </c>
-      <c r="I17" s="51" t="n">
+      <c r="I17" s="46" t="n">
         <v>46</v>
       </c>
-      <c r="J17" s="52" t="n">
+      <c r="J17" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="49" t="inlineStr">
+      <c r="K17" s="44" t="inlineStr">
         <is>
           <t>JA (Kritischer Pfad)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="57" t="inlineStr">
+      <c r="A19" s="52" t="inlineStr">
         <is>
           <t>Gesamte Projektdauer auf dem kritischen Pfad:</t>
         </is>
       </c>
-      <c r="F19" s="58" t="inlineStr">
+      <c r="F19" s="53" t="inlineStr">
         <is>
           <t>46 Arbeitstage (Gesamtpuffer auf kritischem Pfad: 0 Tage | Puffer bei V10: 1 Tag)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="59" t="inlineStr">
-        <is>
-          <t>Formeln &amp; Rechenregeln der Netzplantechnik nach DIN 69900:</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="60" t="inlineStr">
-        <is>
-          <t>1. Vorwärtsrechnung: FEZ = FAZ + Dauer. Bei mehreren Vorgängern gilt für den Nachfolger: FAZ = Maximum aller FEZ der Vorgänger.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="60" t="inlineStr">
-        <is>
-          <t>2. Rückwärtsrechnung: SAZ = SEZ - Dauer. Bei mehreren Nachfolgern gilt für den Vorgänger: SEZ = Minimum aller SAZ der Nachfolger.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="60" t="inlineStr">
-        <is>
-          <t>3. Gesamtpuffer (GP): GP = SAZ - FAZ = SEZ - FEZ. Ein Vorgang mit GP = 0 liegt zwingend auf dem kritischen Pfad!</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="60" t="inlineStr">
-        <is>
-          <t>4. Freier Puffer (FP): FP = min(FAZ_Nachfolger) - FEZ. Gibt an, um wie viel ein Vorgang verzögert werden kann, ohne den FAZ des Nachfolgers zu beeinflussen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="60" t="inlineStr">
-        <is>
-          <t>5. Parallele Vorgänge: V10 (Entsorgung) und V11 (Montage) starten beide nach V9 (FAZ = 39). V11 bestimmt den kritischen Pfad (D=3, FEZ=42). V10 (D=2, FEZ=41) besitzt 1 Tag Puffer (GP=1, FP=1).</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A22:K22"/>
+  <mergeCells count="3">
     <mergeCell ref="F19:K19"/>
-    <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A24:K24"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A23:K23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>